<commit_message>
Class progress per event, blank time is 10 seconds, 7주차_영단어 template
- Event detail shows every class: ✓ with the last day, class accuracy and number of runs; △ when the run ended
  before half the words; or 아직. The class chosen for 대기실 열기 is outlined, with a note when it has already
  had the quiz. The event list shows the same classes and an N/M반 count instead of a raw run count.
- A blank 시간(초) cell now means 10 seconds (단답형 still at least 20); the templates leave it blank.
- [템플릿 받기] downloads 7주차_영단어.xlsx: a teacher's Lesson 7 list (44 words) with the current guide, built by
  make_vocab_template.py like the other examples.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/classeum-vocab-week1.xlsx
+++ b/public/templates/classeum-vocab-week1.xlsx
@@ -586,7 +586,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>시간(초) (선택): 칸마다 10초가 미리 들어 있어요. 단어마다 바꿀 수 있고, 지우면 15초입니다.</t>
+          <t>시간(초) (선택): 비워 두면 10초예요. 오래 걸리는 단어만 숫자를 쓰세요.</t>
         </is>
       </c>
     </row>
@@ -780,9 +780,7 @@
           <t>나는 방과 후에 도서관에서 공부한다.</t>
         </is>
       </c>
-      <c r="G2" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G2" s="6" t="n"/>
       <c r="H2" s="8" t="n"/>
       <c r="I2" s="8" t="n"/>
       <c r="J2" s="6" t="n"/>
@@ -819,9 +817,7 @@
           <t>네 펜 좀 빌려도 될까?</t>
         </is>
       </c>
-      <c r="G3" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G3" s="6" t="n"/>
       <c r="H3" s="8" t="n"/>
       <c r="I3" s="8" t="n"/>
       <c r="J3" s="6" t="n"/>
@@ -858,9 +854,7 @@
           <t>지우개 좀 빌려줄래?</t>
         </is>
       </c>
-      <c r="G4" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G4" s="6" t="n"/>
       <c r="H4" s="8" t="n"/>
       <c r="I4" s="8" t="n"/>
       <c r="J4" s="6" t="n"/>
@@ -893,9 +887,7 @@
           <t>내가 가장 좋아하는 과목은 수학이다.</t>
         </is>
       </c>
-      <c r="G5" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G5" s="6" t="n"/>
       <c r="H5" s="8" t="n"/>
       <c r="I5" s="8" t="n"/>
       <c r="J5" s="6" t="n"/>
@@ -932,9 +924,7 @@
           <t>도서관에서는 조용히 해 주세요.</t>
         </is>
       </c>
-      <c r="G6" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G6" s="6" t="n"/>
       <c r="H6" s="8" t="n"/>
       <c r="I6" s="8" t="n"/>
       <c r="J6" s="6" t="n"/>
@@ -971,9 +961,7 @@
           <t>나는 월요일에 일찍 일어난다.</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G7" s="6" t="n"/>
       <c r="H7" s="8" t="n"/>
       <c r="I7" s="8" t="n"/>
       <c r="J7" s="6" t="n"/>
@@ -1010,9 +998,7 @@
           <t>수업에 늦지 마.</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G8" s="6" t="n"/>
       <c r="H8" s="8" t="n"/>
       <c r="I8" s="8" t="n"/>
       <c r="J8" s="6" t="n"/>
@@ -1045,9 +1031,7 @@
           <t>나는 숙제를 끝냈다.</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G9" s="6" t="n"/>
       <c r="H9" s="8" t="n"/>
       <c r="I9" s="8" t="n"/>
       <c r="J9" s="6" t="n"/>
@@ -1072,9 +1056,7 @@
       <c r="D10" s="6" t="n"/>
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="7" t="n"/>
-      <c r="G10" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G10" s="6" t="n"/>
       <c r="H10" s="8" t="n"/>
       <c r="I10" s="8" t="n"/>
       <c r="J10" s="6" t="n"/>
@@ -1099,9 +1081,7 @@
       <c r="D11" s="6" t="n"/>
       <c r="E11" s="7" t="n"/>
       <c r="F11" s="7" t="n"/>
-      <c r="G11" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G11" s="6" t="n"/>
       <c r="H11" s="8" t="n"/>
       <c r="I11" s="8" t="n"/>
       <c r="J11" s="6" t="n"/>
@@ -1134,9 +1114,7 @@
           <t>오늘 수학 시험이 있다.</t>
         </is>
       </c>
-      <c r="G12" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G12" s="6" t="n"/>
       <c r="H12" s="8" t="n"/>
       <c r="I12" s="8" t="n"/>
       <c r="J12" s="6" t="n"/>
@@ -1173,9 +1151,7 @@
           <t>질문 하나 해도 될까요?</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G13" s="6" t="n"/>
       <c r="H13" s="8" t="n"/>
       <c r="I13" s="8" t="n"/>
       <c r="J13" s="6" t="n"/>
@@ -1212,9 +1188,7 @@
           <t>나는 답을 안다.</t>
         </is>
       </c>
-      <c r="G14" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G14" s="6" t="n"/>
       <c r="H14" s="8" t="n"/>
       <c r="I14" s="8" t="n"/>
       <c r="J14" s="6" t="n"/>
@@ -1243,9 +1217,7 @@
       </c>
       <c r="E15" s="7" t="n"/>
       <c r="F15" s="7" t="n"/>
-      <c r="G15" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G15" s="6" t="n"/>
       <c r="H15" s="8" t="n"/>
       <c r="I15" s="8" t="n"/>
       <c r="J15" s="6" t="n"/>
@@ -1274,9 +1246,7 @@
       </c>
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="7" t="n"/>
-      <c r="G16" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G16" s="6" t="n"/>
       <c r="H16" s="8" t="n"/>
       <c r="I16" s="8" t="n"/>
       <c r="J16" s="6" t="n"/>
@@ -1305,9 +1275,7 @@
       </c>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="7" t="n"/>
-      <c r="G17" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G17" s="6" t="n"/>
       <c r="H17" s="8" t="n"/>
       <c r="I17" s="8" t="n"/>
       <c r="J17" s="6" t="n"/>
@@ -1336,9 +1304,7 @@
       </c>
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="7" t="n"/>
-      <c r="G18" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G18" s="6" t="n"/>
       <c r="H18" s="8" t="n"/>
       <c r="I18" s="8" t="n"/>
       <c r="J18" s="6" t="n"/>
@@ -1371,9 +1337,7 @@
           <t>나는 매일 영어를 연습한다.</t>
         </is>
       </c>
-      <c r="G19" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G19" s="6" t="n"/>
       <c r="H19" s="8" t="n"/>
       <c r="I19" s="8" t="n"/>
       <c r="J19" s="6" t="n"/>
@@ -1402,9 +1366,7 @@
       </c>
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="7" t="n"/>
-      <c r="G20" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G20" s="6" t="n"/>
       <c r="H20" s="8" t="n"/>
       <c r="I20" s="8" t="n"/>
       <c r="J20" s="6" t="n"/>
@@ -1437,3842 +1399,2403 @@
           <t>쉬는 시간에 축구하자.</t>
         </is>
       </c>
-      <c r="G21" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G21" s="6" t="n"/>
       <c r="H21" s="8" t="n"/>
       <c r="I21" s="8" t="n"/>
       <c r="J21" s="6" t="n"/>
       <c r="K21" s="8" t="n"/>
     </row>
     <row r="22">
-      <c r="G22" t="n">
-        <v>10</v>
-      </c>
       <c r="H22" s="9" t="n"/>
       <c r="I22" s="9" t="n"/>
       <c r="K22" s="9" t="n"/>
     </row>
     <row r="23">
-      <c r="G23" t="n">
-        <v>10</v>
-      </c>
       <c r="H23" s="9" t="n"/>
       <c r="I23" s="9" t="n"/>
       <c r="K23" s="9" t="n"/>
     </row>
     <row r="24">
-      <c r="G24" t="n">
-        <v>10</v>
-      </c>
       <c r="H24" s="9" t="n"/>
       <c r="I24" s="9" t="n"/>
       <c r="K24" s="9" t="n"/>
     </row>
     <row r="25">
-      <c r="G25" t="n">
-        <v>10</v>
-      </c>
       <c r="H25" s="9" t="n"/>
       <c r="I25" s="9" t="n"/>
       <c r="K25" s="9" t="n"/>
     </row>
     <row r="26">
-      <c r="G26" t="n">
-        <v>10</v>
-      </c>
       <c r="H26" s="9" t="n"/>
       <c r="I26" s="9" t="n"/>
       <c r="K26" s="9" t="n"/>
     </row>
     <row r="27">
-      <c r="G27" t="n">
-        <v>10</v>
-      </c>
       <c r="H27" s="9" t="n"/>
       <c r="I27" s="9" t="n"/>
       <c r="K27" s="9" t="n"/>
     </row>
     <row r="28">
-      <c r="G28" t="n">
-        <v>10</v>
-      </c>
       <c r="H28" s="9" t="n"/>
       <c r="I28" s="9" t="n"/>
       <c r="K28" s="9" t="n"/>
     </row>
     <row r="29">
-      <c r="G29" t="n">
-        <v>10</v>
-      </c>
       <c r="H29" s="9" t="n"/>
       <c r="I29" s="9" t="n"/>
       <c r="K29" s="9" t="n"/>
     </row>
     <row r="30">
-      <c r="G30" t="n">
-        <v>10</v>
-      </c>
       <c r="H30" s="9" t="n"/>
       <c r="I30" s="9" t="n"/>
       <c r="K30" s="9" t="n"/>
     </row>
     <row r="31">
-      <c r="G31" t="n">
-        <v>10</v>
-      </c>
       <c r="H31" s="9" t="n"/>
       <c r="I31" s="9" t="n"/>
       <c r="K31" s="9" t="n"/>
     </row>
     <row r="32">
-      <c r="G32" t="n">
-        <v>10</v>
-      </c>
       <c r="H32" s="9" t="n"/>
       <c r="I32" s="9" t="n"/>
       <c r="K32" s="9" t="n"/>
     </row>
     <row r="33">
-      <c r="G33" t="n">
-        <v>10</v>
-      </c>
       <c r="H33" s="9" t="n"/>
       <c r="I33" s="9" t="n"/>
       <c r="K33" s="9" t="n"/>
     </row>
     <row r="34">
-      <c r="G34" t="n">
-        <v>10</v>
-      </c>
       <c r="H34" s="9" t="n"/>
       <c r="I34" s="9" t="n"/>
       <c r="K34" s="9" t="n"/>
     </row>
     <row r="35">
-      <c r="G35" t="n">
-        <v>10</v>
-      </c>
       <c r="H35" s="9" t="n"/>
       <c r="I35" s="9" t="n"/>
       <c r="K35" s="9" t="n"/>
     </row>
     <row r="36">
-      <c r="G36" t="n">
-        <v>10</v>
-      </c>
       <c r="H36" s="9" t="n"/>
       <c r="I36" s="9" t="n"/>
       <c r="K36" s="9" t="n"/>
     </row>
     <row r="37">
-      <c r="G37" t="n">
-        <v>10</v>
-      </c>
       <c r="H37" s="9" t="n"/>
       <c r="I37" s="9" t="n"/>
       <c r="K37" s="9" t="n"/>
     </row>
     <row r="38">
-      <c r="G38" t="n">
-        <v>10</v>
-      </c>
       <c r="H38" s="9" t="n"/>
       <c r="I38" s="9" t="n"/>
       <c r="K38" s="9" t="n"/>
     </row>
     <row r="39">
-      <c r="G39" t="n">
-        <v>10</v>
-      </c>
       <c r="H39" s="9" t="n"/>
       <c r="I39" s="9" t="n"/>
       <c r="K39" s="9" t="n"/>
     </row>
     <row r="40">
-      <c r="G40" t="n">
-        <v>10</v>
-      </c>
       <c r="H40" s="9" t="n"/>
       <c r="I40" s="9" t="n"/>
       <c r="K40" s="9" t="n"/>
     </row>
     <row r="41">
-      <c r="G41" t="n">
-        <v>10</v>
-      </c>
       <c r="H41" s="9" t="n"/>
       <c r="I41" s="9" t="n"/>
       <c r="K41" s="9" t="n"/>
     </row>
     <row r="42">
-      <c r="G42" t="n">
-        <v>10</v>
-      </c>
       <c r="H42" s="9" t="n"/>
       <c r="I42" s="9" t="n"/>
       <c r="K42" s="9" t="n"/>
     </row>
     <row r="43">
-      <c r="G43" t="n">
-        <v>10</v>
-      </c>
       <c r="H43" s="9" t="n"/>
       <c r="I43" s="9" t="n"/>
       <c r="K43" s="9" t="n"/>
     </row>
     <row r="44">
-      <c r="G44" t="n">
-        <v>10</v>
-      </c>
       <c r="H44" s="9" t="n"/>
       <c r="I44" s="9" t="n"/>
       <c r="K44" s="9" t="n"/>
     </row>
     <row r="45">
-      <c r="G45" t="n">
-        <v>10</v>
-      </c>
       <c r="H45" s="9" t="n"/>
       <c r="I45" s="9" t="n"/>
       <c r="K45" s="9" t="n"/>
     </row>
     <row r="46">
-      <c r="G46" t="n">
-        <v>10</v>
-      </c>
       <c r="H46" s="9" t="n"/>
       <c r="I46" s="9" t="n"/>
       <c r="K46" s="9" t="n"/>
     </row>
     <row r="47">
-      <c r="G47" t="n">
-        <v>10</v>
-      </c>
       <c r="H47" s="9" t="n"/>
       <c r="I47" s="9" t="n"/>
       <c r="K47" s="9" t="n"/>
     </row>
     <row r="48">
-      <c r="G48" t="n">
-        <v>10</v>
-      </c>
       <c r="H48" s="9" t="n"/>
       <c r="I48" s="9" t="n"/>
       <c r="K48" s="9" t="n"/>
     </row>
     <row r="49">
-      <c r="G49" t="n">
-        <v>10</v>
-      </c>
       <c r="H49" s="9" t="n"/>
       <c r="I49" s="9" t="n"/>
       <c r="K49" s="9" t="n"/>
     </row>
     <row r="50">
-      <c r="G50" t="n">
-        <v>10</v>
-      </c>
       <c r="H50" s="9" t="n"/>
       <c r="I50" s="9" t="n"/>
       <c r="K50" s="9" t="n"/>
     </row>
     <row r="51">
-      <c r="G51" t="n">
-        <v>10</v>
-      </c>
       <c r="H51" s="9" t="n"/>
       <c r="I51" s="9" t="n"/>
       <c r="K51" s="9" t="n"/>
     </row>
     <row r="52">
-      <c r="G52" t="n">
-        <v>10</v>
-      </c>
       <c r="H52" s="9" t="n"/>
       <c r="I52" s="9" t="n"/>
       <c r="K52" s="9" t="n"/>
     </row>
     <row r="53">
-      <c r="G53" t="n">
-        <v>10</v>
-      </c>
       <c r="H53" s="9" t="n"/>
       <c r="I53" s="9" t="n"/>
       <c r="K53" s="9" t="n"/>
     </row>
     <row r="54">
-      <c r="G54" t="n">
-        <v>10</v>
-      </c>
       <c r="H54" s="9" t="n"/>
       <c r="I54" s="9" t="n"/>
       <c r="K54" s="9" t="n"/>
     </row>
     <row r="55">
-      <c r="G55" t="n">
-        <v>10</v>
-      </c>
       <c r="H55" s="9" t="n"/>
       <c r="I55" s="9" t="n"/>
       <c r="K55" s="9" t="n"/>
     </row>
     <row r="56">
-      <c r="G56" t="n">
-        <v>10</v>
-      </c>
       <c r="H56" s="9" t="n"/>
       <c r="I56" s="9" t="n"/>
       <c r="K56" s="9" t="n"/>
     </row>
     <row r="57">
-      <c r="G57" t="n">
-        <v>10</v>
-      </c>
       <c r="H57" s="9" t="n"/>
       <c r="I57" s="9" t="n"/>
       <c r="K57" s="9" t="n"/>
     </row>
     <row r="58">
-      <c r="G58" t="n">
-        <v>10</v>
-      </c>
       <c r="H58" s="9" t="n"/>
       <c r="I58" s="9" t="n"/>
       <c r="K58" s="9" t="n"/>
     </row>
     <row r="59">
-      <c r="G59" t="n">
-        <v>10</v>
-      </c>
       <c r="H59" s="9" t="n"/>
       <c r="I59" s="9" t="n"/>
       <c r="K59" s="9" t="n"/>
     </row>
     <row r="60">
-      <c r="G60" t="n">
-        <v>10</v>
-      </c>
       <c r="H60" s="9" t="n"/>
       <c r="I60" s="9" t="n"/>
       <c r="K60" s="9" t="n"/>
     </row>
     <row r="61">
-      <c r="G61" t="n">
-        <v>10</v>
-      </c>
       <c r="H61" s="9" t="n"/>
       <c r="I61" s="9" t="n"/>
       <c r="K61" s="9" t="n"/>
     </row>
     <row r="62">
-      <c r="G62" t="n">
-        <v>10</v>
-      </c>
       <c r="H62" s="9" t="n"/>
       <c r="I62" s="9" t="n"/>
       <c r="K62" s="9" t="n"/>
     </row>
     <row r="63">
-      <c r="G63" t="n">
-        <v>10</v>
-      </c>
       <c r="H63" s="9" t="n"/>
       <c r="I63" s="9" t="n"/>
       <c r="K63" s="9" t="n"/>
     </row>
     <row r="64">
-      <c r="G64" t="n">
-        <v>10</v>
-      </c>
       <c r="H64" s="9" t="n"/>
       <c r="I64" s="9" t="n"/>
       <c r="K64" s="9" t="n"/>
     </row>
     <row r="65">
-      <c r="G65" t="n">
-        <v>10</v>
-      </c>
       <c r="H65" s="9" t="n"/>
       <c r="I65" s="9" t="n"/>
       <c r="K65" s="9" t="n"/>
     </row>
     <row r="66">
-      <c r="G66" t="n">
-        <v>10</v>
-      </c>
       <c r="H66" s="9" t="n"/>
       <c r="I66" s="9" t="n"/>
       <c r="K66" s="9" t="n"/>
     </row>
     <row r="67">
-      <c r="G67" t="n">
-        <v>10</v>
-      </c>
       <c r="H67" s="9" t="n"/>
       <c r="I67" s="9" t="n"/>
       <c r="K67" s="9" t="n"/>
     </row>
     <row r="68">
-      <c r="G68" t="n">
-        <v>10</v>
-      </c>
       <c r="H68" s="9" t="n"/>
       <c r="I68" s="9" t="n"/>
       <c r="K68" s="9" t="n"/>
     </row>
     <row r="69">
-      <c r="G69" t="n">
-        <v>10</v>
-      </c>
       <c r="H69" s="9" t="n"/>
       <c r="I69" s="9" t="n"/>
       <c r="K69" s="9" t="n"/>
     </row>
     <row r="70">
-      <c r="G70" t="n">
-        <v>10</v>
-      </c>
       <c r="H70" s="9" t="n"/>
       <c r="I70" s="9" t="n"/>
       <c r="K70" s="9" t="n"/>
     </row>
     <row r="71">
-      <c r="G71" t="n">
-        <v>10</v>
-      </c>
       <c r="H71" s="9" t="n"/>
       <c r="I71" s="9" t="n"/>
       <c r="K71" s="9" t="n"/>
     </row>
     <row r="72">
-      <c r="G72" t="n">
-        <v>10</v>
-      </c>
       <c r="H72" s="9" t="n"/>
       <c r="I72" s="9" t="n"/>
       <c r="K72" s="9" t="n"/>
     </row>
     <row r="73">
-      <c r="G73" t="n">
-        <v>10</v>
-      </c>
       <c r="H73" s="9" t="n"/>
       <c r="I73" s="9" t="n"/>
       <c r="K73" s="9" t="n"/>
     </row>
     <row r="74">
-      <c r="G74" t="n">
-        <v>10</v>
-      </c>
       <c r="H74" s="9" t="n"/>
       <c r="I74" s="9" t="n"/>
       <c r="K74" s="9" t="n"/>
     </row>
     <row r="75">
-      <c r="G75" t="n">
-        <v>10</v>
-      </c>
       <c r="H75" s="9" t="n"/>
       <c r="I75" s="9" t="n"/>
       <c r="K75" s="9" t="n"/>
     </row>
     <row r="76">
-      <c r="G76" t="n">
-        <v>10</v>
-      </c>
       <c r="H76" s="9" t="n"/>
       <c r="I76" s="9" t="n"/>
       <c r="K76" s="9" t="n"/>
     </row>
     <row r="77">
-      <c r="G77" t="n">
-        <v>10</v>
-      </c>
       <c r="H77" s="9" t="n"/>
       <c r="I77" s="9" t="n"/>
       <c r="K77" s="9" t="n"/>
     </row>
     <row r="78">
-      <c r="G78" t="n">
-        <v>10</v>
-      </c>
       <c r="H78" s="9" t="n"/>
       <c r="I78" s="9" t="n"/>
       <c r="K78" s="9" t="n"/>
     </row>
     <row r="79">
-      <c r="G79" t="n">
-        <v>10</v>
-      </c>
       <c r="H79" s="9" t="n"/>
       <c r="I79" s="9" t="n"/>
       <c r="K79" s="9" t="n"/>
     </row>
     <row r="80">
-      <c r="G80" t="n">
-        <v>10</v>
-      </c>
       <c r="H80" s="9" t="n"/>
       <c r="I80" s="9" t="n"/>
       <c r="K80" s="9" t="n"/>
     </row>
     <row r="81">
-      <c r="G81" t="n">
-        <v>10</v>
-      </c>
       <c r="H81" s="9" t="n"/>
       <c r="I81" s="9" t="n"/>
       <c r="K81" s="9" t="n"/>
     </row>
     <row r="82">
-      <c r="G82" t="n">
-        <v>10</v>
-      </c>
       <c r="H82" s="9" t="n"/>
       <c r="I82" s="9" t="n"/>
       <c r="K82" s="9" t="n"/>
     </row>
     <row r="83">
-      <c r="G83" t="n">
-        <v>10</v>
-      </c>
       <c r="H83" s="9" t="n"/>
       <c r="I83" s="9" t="n"/>
       <c r="K83" s="9" t="n"/>
     </row>
     <row r="84">
-      <c r="G84" t="n">
-        <v>10</v>
-      </c>
       <c r="H84" s="9" t="n"/>
       <c r="I84" s="9" t="n"/>
       <c r="K84" s="9" t="n"/>
     </row>
     <row r="85">
-      <c r="G85" t="n">
-        <v>10</v>
-      </c>
       <c r="H85" s="9" t="n"/>
       <c r="I85" s="9" t="n"/>
       <c r="K85" s="9" t="n"/>
     </row>
     <row r="86">
-      <c r="G86" t="n">
-        <v>10</v>
-      </c>
       <c r="H86" s="9" t="n"/>
       <c r="I86" s="9" t="n"/>
       <c r="K86" s="9" t="n"/>
     </row>
     <row r="87">
-      <c r="G87" t="n">
-        <v>10</v>
-      </c>
       <c r="H87" s="9" t="n"/>
       <c r="I87" s="9" t="n"/>
       <c r="K87" s="9" t="n"/>
     </row>
     <row r="88">
-      <c r="G88" t="n">
-        <v>10</v>
-      </c>
       <c r="H88" s="9" t="n"/>
       <c r="I88" s="9" t="n"/>
       <c r="K88" s="9" t="n"/>
     </row>
     <row r="89">
-      <c r="G89" t="n">
-        <v>10</v>
-      </c>
       <c r="H89" s="9" t="n"/>
       <c r="I89" s="9" t="n"/>
       <c r="K89" s="9" t="n"/>
     </row>
     <row r="90">
-      <c r="G90" t="n">
-        <v>10</v>
-      </c>
       <c r="H90" s="9" t="n"/>
       <c r="I90" s="9" t="n"/>
       <c r="K90" s="9" t="n"/>
     </row>
     <row r="91">
-      <c r="G91" t="n">
-        <v>10</v>
-      </c>
       <c r="H91" s="9" t="n"/>
       <c r="I91" s="9" t="n"/>
       <c r="K91" s="9" t="n"/>
     </row>
     <row r="92">
-      <c r="G92" t="n">
-        <v>10</v>
-      </c>
       <c r="H92" s="9" t="n"/>
       <c r="I92" s="9" t="n"/>
       <c r="K92" s="9" t="n"/>
     </row>
     <row r="93">
-      <c r="G93" t="n">
-        <v>10</v>
-      </c>
       <c r="H93" s="9" t="n"/>
       <c r="I93" s="9" t="n"/>
       <c r="K93" s="9" t="n"/>
     </row>
     <row r="94">
-      <c r="G94" t="n">
-        <v>10</v>
-      </c>
       <c r="H94" s="9" t="n"/>
       <c r="I94" s="9" t="n"/>
       <c r="K94" s="9" t="n"/>
     </row>
     <row r="95">
-      <c r="G95" t="n">
-        <v>10</v>
-      </c>
       <c r="H95" s="9" t="n"/>
       <c r="I95" s="9" t="n"/>
       <c r="K95" s="9" t="n"/>
     </row>
     <row r="96">
-      <c r="G96" t="n">
-        <v>10</v>
-      </c>
       <c r="H96" s="9" t="n"/>
       <c r="I96" s="9" t="n"/>
       <c r="K96" s="9" t="n"/>
     </row>
     <row r="97">
-      <c r="G97" t="n">
-        <v>10</v>
-      </c>
       <c r="H97" s="9" t="n"/>
       <c r="I97" s="9" t="n"/>
       <c r="K97" s="9" t="n"/>
     </row>
     <row r="98">
-      <c r="G98" t="n">
-        <v>10</v>
-      </c>
       <c r="H98" s="9" t="n"/>
       <c r="I98" s="9" t="n"/>
       <c r="K98" s="9" t="n"/>
     </row>
     <row r="99">
-      <c r="G99" t="n">
-        <v>10</v>
-      </c>
       <c r="H99" s="9" t="n"/>
       <c r="I99" s="9" t="n"/>
       <c r="K99" s="9" t="n"/>
     </row>
     <row r="100">
-      <c r="G100" t="n">
-        <v>10</v>
-      </c>
       <c r="H100" s="9" t="n"/>
       <c r="I100" s="9" t="n"/>
       <c r="K100" s="9" t="n"/>
     </row>
     <row r="101">
-      <c r="G101" t="n">
-        <v>10</v>
-      </c>
       <c r="H101" s="9" t="n"/>
       <c r="I101" s="9" t="n"/>
       <c r="K101" s="9" t="n"/>
     </row>
     <row r="102">
-      <c r="G102" t="n">
-        <v>10</v>
-      </c>
       <c r="H102" s="9" t="n"/>
       <c r="I102" s="9" t="n"/>
       <c r="K102" s="9" t="n"/>
     </row>
     <row r="103">
-      <c r="G103" t="n">
-        <v>10</v>
-      </c>
       <c r="H103" s="9" t="n"/>
       <c r="I103" s="9" t="n"/>
       <c r="K103" s="9" t="n"/>
     </row>
     <row r="104">
-      <c r="G104" t="n">
-        <v>10</v>
-      </c>
       <c r="H104" s="9" t="n"/>
       <c r="I104" s="9" t="n"/>
       <c r="K104" s="9" t="n"/>
     </row>
     <row r="105">
-      <c r="G105" t="n">
-        <v>10</v>
-      </c>
       <c r="H105" s="9" t="n"/>
       <c r="I105" s="9" t="n"/>
       <c r="K105" s="9" t="n"/>
     </row>
     <row r="106">
-      <c r="G106" t="n">
-        <v>10</v>
-      </c>
       <c r="H106" s="9" t="n"/>
       <c r="I106" s="9" t="n"/>
       <c r="K106" s="9" t="n"/>
     </row>
     <row r="107">
-      <c r="G107" t="n">
-        <v>10</v>
-      </c>
       <c r="H107" s="9" t="n"/>
       <c r="I107" s="9" t="n"/>
       <c r="K107" s="9" t="n"/>
     </row>
     <row r="108">
-      <c r="G108" t="n">
-        <v>10</v>
-      </c>
       <c r="H108" s="9" t="n"/>
       <c r="I108" s="9" t="n"/>
       <c r="K108" s="9" t="n"/>
     </row>
     <row r="109">
-      <c r="G109" t="n">
-        <v>10</v>
-      </c>
       <c r="H109" s="9" t="n"/>
       <c r="I109" s="9" t="n"/>
       <c r="K109" s="9" t="n"/>
     </row>
     <row r="110">
-      <c r="G110" t="n">
-        <v>10</v>
-      </c>
       <c r="H110" s="9" t="n"/>
       <c r="I110" s="9" t="n"/>
       <c r="K110" s="9" t="n"/>
     </row>
     <row r="111">
-      <c r="G111" t="n">
-        <v>10</v>
-      </c>
       <c r="H111" s="9" t="n"/>
       <c r="I111" s="9" t="n"/>
       <c r="K111" s="9" t="n"/>
     </row>
     <row r="112">
-      <c r="G112" t="n">
-        <v>10</v>
-      </c>
       <c r="H112" s="9" t="n"/>
       <c r="I112" s="9" t="n"/>
       <c r="K112" s="9" t="n"/>
     </row>
     <row r="113">
-      <c r="G113" t="n">
-        <v>10</v>
-      </c>
       <c r="H113" s="9" t="n"/>
       <c r="I113" s="9" t="n"/>
       <c r="K113" s="9" t="n"/>
     </row>
     <row r="114">
-      <c r="G114" t="n">
-        <v>10</v>
-      </c>
       <c r="H114" s="9" t="n"/>
       <c r="I114" s="9" t="n"/>
       <c r="K114" s="9" t="n"/>
     </row>
     <row r="115">
-      <c r="G115" t="n">
-        <v>10</v>
-      </c>
       <c r="H115" s="9" t="n"/>
       <c r="I115" s="9" t="n"/>
       <c r="K115" s="9" t="n"/>
     </row>
     <row r="116">
-      <c r="G116" t="n">
-        <v>10</v>
-      </c>
       <c r="H116" s="9" t="n"/>
       <c r="I116" s="9" t="n"/>
       <c r="K116" s="9" t="n"/>
     </row>
     <row r="117">
-      <c r="G117" t="n">
-        <v>10</v>
-      </c>
       <c r="H117" s="9" t="n"/>
       <c r="I117" s="9" t="n"/>
       <c r="K117" s="9" t="n"/>
     </row>
     <row r="118">
-      <c r="G118" t="n">
-        <v>10</v>
-      </c>
       <c r="H118" s="9" t="n"/>
       <c r="I118" s="9" t="n"/>
       <c r="K118" s="9" t="n"/>
     </row>
     <row r="119">
-      <c r="G119" t="n">
-        <v>10</v>
-      </c>
       <c r="H119" s="9" t="n"/>
       <c r="I119" s="9" t="n"/>
       <c r="K119" s="9" t="n"/>
     </row>
     <row r="120">
-      <c r="G120" t="n">
-        <v>10</v>
-      </c>
       <c r="H120" s="9" t="n"/>
       <c r="I120" s="9" t="n"/>
       <c r="K120" s="9" t="n"/>
     </row>
     <row r="121">
-      <c r="G121" t="n">
-        <v>10</v>
-      </c>
       <c r="H121" s="9" t="n"/>
       <c r="I121" s="9" t="n"/>
       <c r="K121" s="9" t="n"/>
     </row>
     <row r="122">
-      <c r="G122" t="n">
-        <v>10</v>
-      </c>
       <c r="H122" s="9" t="n"/>
       <c r="I122" s="9" t="n"/>
       <c r="K122" s="9" t="n"/>
     </row>
     <row r="123">
-      <c r="G123" t="n">
-        <v>10</v>
-      </c>
       <c r="H123" s="9" t="n"/>
       <c r="I123" s="9" t="n"/>
       <c r="K123" s="9" t="n"/>
     </row>
     <row r="124">
-      <c r="G124" t="n">
-        <v>10</v>
-      </c>
       <c r="H124" s="9" t="n"/>
       <c r="I124" s="9" t="n"/>
       <c r="K124" s="9" t="n"/>
     </row>
     <row r="125">
-      <c r="G125" t="n">
-        <v>10</v>
-      </c>
       <c r="H125" s="9" t="n"/>
       <c r="I125" s="9" t="n"/>
       <c r="K125" s="9" t="n"/>
     </row>
     <row r="126">
-      <c r="G126" t="n">
-        <v>10</v>
-      </c>
       <c r="H126" s="9" t="n"/>
       <c r="I126" s="9" t="n"/>
       <c r="K126" s="9" t="n"/>
     </row>
     <row r="127">
-      <c r="G127" t="n">
-        <v>10</v>
-      </c>
       <c r="H127" s="9" t="n"/>
       <c r="I127" s="9" t="n"/>
       <c r="K127" s="9" t="n"/>
     </row>
     <row r="128">
-      <c r="G128" t="n">
-        <v>10</v>
-      </c>
       <c r="H128" s="9" t="n"/>
       <c r="I128" s="9" t="n"/>
       <c r="K128" s="9" t="n"/>
     </row>
     <row r="129">
-      <c r="G129" t="n">
-        <v>10</v>
-      </c>
       <c r="H129" s="9" t="n"/>
       <c r="I129" s="9" t="n"/>
       <c r="K129" s="9" t="n"/>
     </row>
     <row r="130">
-      <c r="G130" t="n">
-        <v>10</v>
-      </c>
       <c r="H130" s="9" t="n"/>
       <c r="I130" s="9" t="n"/>
       <c r="K130" s="9" t="n"/>
     </row>
     <row r="131">
-      <c r="G131" t="n">
-        <v>10</v>
-      </c>
       <c r="H131" s="9" t="n"/>
       <c r="I131" s="9" t="n"/>
       <c r="K131" s="9" t="n"/>
     </row>
     <row r="132">
-      <c r="G132" t="n">
-        <v>10</v>
-      </c>
       <c r="H132" s="9" t="n"/>
       <c r="I132" s="9" t="n"/>
       <c r="K132" s="9" t="n"/>
     </row>
     <row r="133">
-      <c r="G133" t="n">
-        <v>10</v>
-      </c>
       <c r="H133" s="9" t="n"/>
       <c r="I133" s="9" t="n"/>
       <c r="K133" s="9" t="n"/>
     </row>
     <row r="134">
-      <c r="G134" t="n">
-        <v>10</v>
-      </c>
       <c r="H134" s="9" t="n"/>
       <c r="I134" s="9" t="n"/>
       <c r="K134" s="9" t="n"/>
     </row>
     <row r="135">
-      <c r="G135" t="n">
-        <v>10</v>
-      </c>
       <c r="H135" s="9" t="n"/>
       <c r="I135" s="9" t="n"/>
       <c r="K135" s="9" t="n"/>
     </row>
     <row r="136">
-      <c r="G136" t="n">
-        <v>10</v>
-      </c>
       <c r="H136" s="9" t="n"/>
       <c r="I136" s="9" t="n"/>
       <c r="K136" s="9" t="n"/>
     </row>
     <row r="137">
-      <c r="G137" t="n">
-        <v>10</v>
-      </c>
       <c r="H137" s="9" t="n"/>
       <c r="I137" s="9" t="n"/>
       <c r="K137" s="9" t="n"/>
     </row>
     <row r="138">
-      <c r="G138" t="n">
-        <v>10</v>
-      </c>
       <c r="H138" s="9" t="n"/>
       <c r="I138" s="9" t="n"/>
       <c r="K138" s="9" t="n"/>
     </row>
     <row r="139">
-      <c r="G139" t="n">
-        <v>10</v>
-      </c>
       <c r="H139" s="9" t="n"/>
       <c r="I139" s="9" t="n"/>
       <c r="K139" s="9" t="n"/>
     </row>
     <row r="140">
-      <c r="G140" t="n">
-        <v>10</v>
-      </c>
       <c r="H140" s="9" t="n"/>
       <c r="I140" s="9" t="n"/>
       <c r="K140" s="9" t="n"/>
     </row>
     <row r="141">
-      <c r="G141" t="n">
-        <v>10</v>
-      </c>
       <c r="H141" s="9" t="n"/>
       <c r="I141" s="9" t="n"/>
       <c r="K141" s="9" t="n"/>
     </row>
     <row r="142">
-      <c r="G142" t="n">
-        <v>10</v>
-      </c>
       <c r="H142" s="9" t="n"/>
       <c r="I142" s="9" t="n"/>
       <c r="K142" s="9" t="n"/>
     </row>
     <row r="143">
-      <c r="G143" t="n">
-        <v>10</v>
-      </c>
       <c r="H143" s="9" t="n"/>
       <c r="I143" s="9" t="n"/>
       <c r="K143" s="9" t="n"/>
     </row>
     <row r="144">
-      <c r="G144" t="n">
-        <v>10</v>
-      </c>
       <c r="H144" s="9" t="n"/>
       <c r="I144" s="9" t="n"/>
       <c r="K144" s="9" t="n"/>
     </row>
     <row r="145">
-      <c r="G145" t="n">
-        <v>10</v>
-      </c>
       <c r="H145" s="9" t="n"/>
       <c r="I145" s="9" t="n"/>
       <c r="K145" s="9" t="n"/>
     </row>
     <row r="146">
-      <c r="G146" t="n">
-        <v>10</v>
-      </c>
       <c r="H146" s="9" t="n"/>
       <c r="I146" s="9" t="n"/>
       <c r="K146" s="9" t="n"/>
     </row>
     <row r="147">
-      <c r="G147" t="n">
-        <v>10</v>
-      </c>
       <c r="H147" s="9" t="n"/>
       <c r="I147" s="9" t="n"/>
       <c r="K147" s="9" t="n"/>
     </row>
     <row r="148">
-      <c r="G148" t="n">
-        <v>10</v>
-      </c>
       <c r="H148" s="9" t="n"/>
       <c r="I148" s="9" t="n"/>
       <c r="K148" s="9" t="n"/>
     </row>
     <row r="149">
-      <c r="G149" t="n">
-        <v>10</v>
-      </c>
       <c r="H149" s="9" t="n"/>
       <c r="I149" s="9" t="n"/>
       <c r="K149" s="9" t="n"/>
     </row>
     <row r="150">
-      <c r="G150" t="n">
-        <v>10</v>
-      </c>
       <c r="H150" s="9" t="n"/>
       <c r="I150" s="9" t="n"/>
       <c r="K150" s="9" t="n"/>
     </row>
     <row r="151">
-      <c r="G151" t="n">
-        <v>10</v>
-      </c>
       <c r="H151" s="9" t="n"/>
       <c r="I151" s="9" t="n"/>
       <c r="K151" s="9" t="n"/>
     </row>
     <row r="152">
-      <c r="G152" t="n">
-        <v>10</v>
-      </c>
       <c r="H152" s="9" t="n"/>
       <c r="I152" s="9" t="n"/>
       <c r="K152" s="9" t="n"/>
     </row>
     <row r="153">
-      <c r="G153" t="n">
-        <v>10</v>
-      </c>
       <c r="H153" s="9" t="n"/>
       <c r="I153" s="9" t="n"/>
       <c r="K153" s="9" t="n"/>
     </row>
     <row r="154">
-      <c r="G154" t="n">
-        <v>10</v>
-      </c>
       <c r="H154" s="9" t="n"/>
       <c r="I154" s="9" t="n"/>
       <c r="K154" s="9" t="n"/>
     </row>
     <row r="155">
-      <c r="G155" t="n">
-        <v>10</v>
-      </c>
       <c r="H155" s="9" t="n"/>
       <c r="I155" s="9" t="n"/>
       <c r="K155" s="9" t="n"/>
     </row>
     <row r="156">
-      <c r="G156" t="n">
-        <v>10</v>
-      </c>
       <c r="H156" s="9" t="n"/>
       <c r="I156" s="9" t="n"/>
       <c r="K156" s="9" t="n"/>
     </row>
     <row r="157">
-      <c r="G157" t="n">
-        <v>10</v>
-      </c>
       <c r="H157" s="9" t="n"/>
       <c r="I157" s="9" t="n"/>
       <c r="K157" s="9" t="n"/>
     </row>
     <row r="158">
-      <c r="G158" t="n">
-        <v>10</v>
-      </c>
       <c r="H158" s="9" t="n"/>
       <c r="I158" s="9" t="n"/>
       <c r="K158" s="9" t="n"/>
     </row>
     <row r="159">
-      <c r="G159" t="n">
-        <v>10</v>
-      </c>
       <c r="H159" s="9" t="n"/>
       <c r="I159" s="9" t="n"/>
       <c r="K159" s="9" t="n"/>
     </row>
     <row r="160">
-      <c r="G160" t="n">
-        <v>10</v>
-      </c>
       <c r="H160" s="9" t="n"/>
       <c r="I160" s="9" t="n"/>
       <c r="K160" s="9" t="n"/>
     </row>
     <row r="161">
-      <c r="G161" t="n">
-        <v>10</v>
-      </c>
       <c r="H161" s="9" t="n"/>
       <c r="I161" s="9" t="n"/>
       <c r="K161" s="9" t="n"/>
     </row>
     <row r="162">
-      <c r="G162" t="n">
-        <v>10</v>
-      </c>
       <c r="H162" s="9" t="n"/>
       <c r="I162" s="9" t="n"/>
       <c r="K162" s="9" t="n"/>
     </row>
     <row r="163">
-      <c r="G163" t="n">
-        <v>10</v>
-      </c>
       <c r="H163" s="9" t="n"/>
       <c r="I163" s="9" t="n"/>
       <c r="K163" s="9" t="n"/>
     </row>
     <row r="164">
-      <c r="G164" t="n">
-        <v>10</v>
-      </c>
       <c r="H164" s="9" t="n"/>
       <c r="I164" s="9" t="n"/>
       <c r="K164" s="9" t="n"/>
     </row>
     <row r="165">
-      <c r="G165" t="n">
-        <v>10</v>
-      </c>
       <c r="H165" s="9" t="n"/>
       <c r="I165" s="9" t="n"/>
       <c r="K165" s="9" t="n"/>
     </row>
     <row r="166">
-      <c r="G166" t="n">
-        <v>10</v>
-      </c>
       <c r="H166" s="9" t="n"/>
       <c r="I166" s="9" t="n"/>
       <c r="K166" s="9" t="n"/>
     </row>
     <row r="167">
-      <c r="G167" t="n">
-        <v>10</v>
-      </c>
       <c r="H167" s="9" t="n"/>
       <c r="I167" s="9" t="n"/>
       <c r="K167" s="9" t="n"/>
     </row>
     <row r="168">
-      <c r="G168" t="n">
-        <v>10</v>
-      </c>
       <c r="H168" s="9" t="n"/>
       <c r="I168" s="9" t="n"/>
       <c r="K168" s="9" t="n"/>
     </row>
     <row r="169">
-      <c r="G169" t="n">
-        <v>10</v>
-      </c>
       <c r="H169" s="9" t="n"/>
       <c r="I169" s="9" t="n"/>
       <c r="K169" s="9" t="n"/>
     </row>
     <row r="170">
-      <c r="G170" t="n">
-        <v>10</v>
-      </c>
       <c r="H170" s="9" t="n"/>
       <c r="I170" s="9" t="n"/>
       <c r="K170" s="9" t="n"/>
     </row>
     <row r="171">
-      <c r="G171" t="n">
-        <v>10</v>
-      </c>
       <c r="H171" s="9" t="n"/>
       <c r="I171" s="9" t="n"/>
       <c r="K171" s="9" t="n"/>
     </row>
     <row r="172">
-      <c r="G172" t="n">
-        <v>10</v>
-      </c>
       <c r="H172" s="9" t="n"/>
       <c r="I172" s="9" t="n"/>
       <c r="K172" s="9" t="n"/>
     </row>
     <row r="173">
-      <c r="G173" t="n">
-        <v>10</v>
-      </c>
       <c r="H173" s="9" t="n"/>
       <c r="I173" s="9" t="n"/>
       <c r="K173" s="9" t="n"/>
     </row>
     <row r="174">
-      <c r="G174" t="n">
-        <v>10</v>
-      </c>
       <c r="H174" s="9" t="n"/>
       <c r="I174" s="9" t="n"/>
       <c r="K174" s="9" t="n"/>
     </row>
     <row r="175">
-      <c r="G175" t="n">
-        <v>10</v>
-      </c>
       <c r="H175" s="9" t="n"/>
       <c r="I175" s="9" t="n"/>
       <c r="K175" s="9" t="n"/>
     </row>
     <row r="176">
-      <c r="G176" t="n">
-        <v>10</v>
-      </c>
       <c r="H176" s="9" t="n"/>
       <c r="I176" s="9" t="n"/>
       <c r="K176" s="9" t="n"/>
     </row>
     <row r="177">
-      <c r="G177" t="n">
-        <v>10</v>
-      </c>
       <c r="H177" s="9" t="n"/>
       <c r="I177" s="9" t="n"/>
       <c r="K177" s="9" t="n"/>
     </row>
     <row r="178">
-      <c r="G178" t="n">
-        <v>10</v>
-      </c>
       <c r="H178" s="9" t="n"/>
       <c r="I178" s="9" t="n"/>
       <c r="K178" s="9" t="n"/>
     </row>
     <row r="179">
-      <c r="G179" t="n">
-        <v>10</v>
-      </c>
       <c r="H179" s="9" t="n"/>
       <c r="I179" s="9" t="n"/>
       <c r="K179" s="9" t="n"/>
     </row>
     <row r="180">
-      <c r="G180" t="n">
-        <v>10</v>
-      </c>
       <c r="H180" s="9" t="n"/>
       <c r="I180" s="9" t="n"/>
       <c r="K180" s="9" t="n"/>
     </row>
     <row r="181">
-      <c r="G181" t="n">
-        <v>10</v>
-      </c>
       <c r="H181" s="9" t="n"/>
       <c r="I181" s="9" t="n"/>
       <c r="K181" s="9" t="n"/>
     </row>
     <row r="182">
-      <c r="G182" t="n">
-        <v>10</v>
-      </c>
       <c r="H182" s="9" t="n"/>
       <c r="I182" s="9" t="n"/>
       <c r="K182" s="9" t="n"/>
     </row>
     <row r="183">
-      <c r="G183" t="n">
-        <v>10</v>
-      </c>
       <c r="H183" s="9" t="n"/>
       <c r="I183" s="9" t="n"/>
       <c r="K183" s="9" t="n"/>
     </row>
     <row r="184">
-      <c r="G184" t="n">
-        <v>10</v>
-      </c>
       <c r="H184" s="9" t="n"/>
       <c r="I184" s="9" t="n"/>
       <c r="K184" s="9" t="n"/>
     </row>
     <row r="185">
-      <c r="G185" t="n">
-        <v>10</v>
-      </c>
       <c r="H185" s="9" t="n"/>
       <c r="I185" s="9" t="n"/>
       <c r="K185" s="9" t="n"/>
     </row>
     <row r="186">
-      <c r="G186" t="n">
-        <v>10</v>
-      </c>
       <c r="H186" s="9" t="n"/>
       <c r="I186" s="9" t="n"/>
       <c r="K186" s="9" t="n"/>
     </row>
     <row r="187">
-      <c r="G187" t="n">
-        <v>10</v>
-      </c>
       <c r="H187" s="9" t="n"/>
       <c r="I187" s="9" t="n"/>
       <c r="K187" s="9" t="n"/>
     </row>
     <row r="188">
-      <c r="G188" t="n">
-        <v>10</v>
-      </c>
       <c r="H188" s="9" t="n"/>
       <c r="I188" s="9" t="n"/>
       <c r="K188" s="9" t="n"/>
     </row>
     <row r="189">
-      <c r="G189" t="n">
-        <v>10</v>
-      </c>
       <c r="H189" s="9" t="n"/>
       <c r="I189" s="9" t="n"/>
       <c r="K189" s="9" t="n"/>
     </row>
     <row r="190">
-      <c r="G190" t="n">
-        <v>10</v>
-      </c>
       <c r="H190" s="9" t="n"/>
       <c r="I190" s="9" t="n"/>
       <c r="K190" s="9" t="n"/>
     </row>
     <row r="191">
-      <c r="G191" t="n">
-        <v>10</v>
-      </c>
       <c r="H191" s="9" t="n"/>
       <c r="I191" s="9" t="n"/>
       <c r="K191" s="9" t="n"/>
     </row>
     <row r="192">
-      <c r="G192" t="n">
-        <v>10</v>
-      </c>
       <c r="H192" s="9" t="n"/>
       <c r="I192" s="9" t="n"/>
       <c r="K192" s="9" t="n"/>
     </row>
     <row r="193">
-      <c r="G193" t="n">
-        <v>10</v>
-      </c>
       <c r="H193" s="9" t="n"/>
       <c r="I193" s="9" t="n"/>
       <c r="K193" s="9" t="n"/>
     </row>
     <row r="194">
-      <c r="G194" t="n">
-        <v>10</v>
-      </c>
       <c r="H194" s="9" t="n"/>
       <c r="I194" s="9" t="n"/>
       <c r="K194" s="9" t="n"/>
     </row>
     <row r="195">
-      <c r="G195" t="n">
-        <v>10</v>
-      </c>
       <c r="H195" s="9" t="n"/>
       <c r="I195" s="9" t="n"/>
       <c r="K195" s="9" t="n"/>
     </row>
     <row r="196">
-      <c r="G196" t="n">
-        <v>10</v>
-      </c>
       <c r="H196" s="9" t="n"/>
       <c r="I196" s="9" t="n"/>
       <c r="K196" s="9" t="n"/>
     </row>
     <row r="197">
-      <c r="G197" t="n">
-        <v>10</v>
-      </c>
       <c r="H197" s="9" t="n"/>
       <c r="I197" s="9" t="n"/>
       <c r="K197" s="9" t="n"/>
     </row>
     <row r="198">
-      <c r="G198" t="n">
-        <v>10</v>
-      </c>
       <c r="H198" s="9" t="n"/>
       <c r="I198" s="9" t="n"/>
       <c r="K198" s="9" t="n"/>
     </row>
     <row r="199">
-      <c r="G199" t="n">
-        <v>10</v>
-      </c>
       <c r="H199" s="9" t="n"/>
       <c r="I199" s="9" t="n"/>
       <c r="K199" s="9" t="n"/>
     </row>
     <row r="200">
-      <c r="G200" t="n">
-        <v>10</v>
-      </c>
       <c r="H200" s="9" t="n"/>
       <c r="I200" s="9" t="n"/>
       <c r="K200" s="9" t="n"/>
     </row>
     <row r="201">
-      <c r="G201" t="n">
-        <v>10</v>
-      </c>
       <c r="H201" s="9" t="n"/>
       <c r="I201" s="9" t="n"/>
       <c r="K201" s="9" t="n"/>
     </row>
     <row r="202">
-      <c r="G202" t="n">
-        <v>10</v>
-      </c>
       <c r="H202" s="9" t="n"/>
       <c r="I202" s="9" t="n"/>
       <c r="K202" s="9" t="n"/>
     </row>
     <row r="203">
-      <c r="G203" t="n">
-        <v>10</v>
-      </c>
       <c r="H203" s="9" t="n"/>
       <c r="I203" s="9" t="n"/>
       <c r="K203" s="9" t="n"/>
     </row>
     <row r="204">
-      <c r="G204" t="n">
-        <v>10</v>
-      </c>
       <c r="H204" s="9" t="n"/>
       <c r="I204" s="9" t="n"/>
       <c r="K204" s="9" t="n"/>
     </row>
     <row r="205">
-      <c r="G205" t="n">
-        <v>10</v>
-      </c>
       <c r="H205" s="9" t="n"/>
       <c r="I205" s="9" t="n"/>
       <c r="K205" s="9" t="n"/>
     </row>
     <row r="206">
-      <c r="G206" t="n">
-        <v>10</v>
-      </c>
       <c r="H206" s="9" t="n"/>
       <c r="I206" s="9" t="n"/>
       <c r="K206" s="9" t="n"/>
     </row>
     <row r="207">
-      <c r="G207" t="n">
-        <v>10</v>
-      </c>
       <c r="H207" s="9" t="n"/>
       <c r="I207" s="9" t="n"/>
       <c r="K207" s="9" t="n"/>
     </row>
     <row r="208">
-      <c r="G208" t="n">
-        <v>10</v>
-      </c>
       <c r="H208" s="9" t="n"/>
       <c r="I208" s="9" t="n"/>
       <c r="K208" s="9" t="n"/>
     </row>
     <row r="209">
-      <c r="G209" t="n">
-        <v>10</v>
-      </c>
       <c r="H209" s="9" t="n"/>
       <c r="I209" s="9" t="n"/>
       <c r="K209" s="9" t="n"/>
     </row>
     <row r="210">
-      <c r="G210" t="n">
-        <v>10</v>
-      </c>
       <c r="H210" s="9" t="n"/>
       <c r="I210" s="9" t="n"/>
       <c r="K210" s="9" t="n"/>
     </row>
     <row r="211">
-      <c r="G211" t="n">
-        <v>10</v>
-      </c>
       <c r="H211" s="9" t="n"/>
       <c r="I211" s="9" t="n"/>
       <c r="K211" s="9" t="n"/>
     </row>
     <row r="212">
-      <c r="G212" t="n">
-        <v>10</v>
-      </c>
       <c r="H212" s="9" t="n"/>
       <c r="I212" s="9" t="n"/>
       <c r="K212" s="9" t="n"/>
     </row>
     <row r="213">
-      <c r="G213" t="n">
-        <v>10</v>
-      </c>
       <c r="H213" s="9" t="n"/>
       <c r="I213" s="9" t="n"/>
       <c r="K213" s="9" t="n"/>
     </row>
     <row r="214">
-      <c r="G214" t="n">
-        <v>10</v>
-      </c>
       <c r="H214" s="9" t="n"/>
       <c r="I214" s="9" t="n"/>
       <c r="K214" s="9" t="n"/>
     </row>
     <row r="215">
-      <c r="G215" t="n">
-        <v>10</v>
-      </c>
       <c r="H215" s="9" t="n"/>
       <c r="I215" s="9" t="n"/>
       <c r="K215" s="9" t="n"/>
     </row>
     <row r="216">
-      <c r="G216" t="n">
-        <v>10</v>
-      </c>
       <c r="H216" s="9" t="n"/>
       <c r="I216" s="9" t="n"/>
       <c r="K216" s="9" t="n"/>
     </row>
     <row r="217">
-      <c r="G217" t="n">
-        <v>10</v>
-      </c>
       <c r="H217" s="9" t="n"/>
       <c r="I217" s="9" t="n"/>
       <c r="K217" s="9" t="n"/>
     </row>
     <row r="218">
-      <c r="G218" t="n">
-        <v>10</v>
-      </c>
       <c r="H218" s="9" t="n"/>
       <c r="I218" s="9" t="n"/>
       <c r="K218" s="9" t="n"/>
     </row>
     <row r="219">
-      <c r="G219" t="n">
-        <v>10</v>
-      </c>
       <c r="H219" s="9" t="n"/>
       <c r="I219" s="9" t="n"/>
       <c r="K219" s="9" t="n"/>
     </row>
     <row r="220">
-      <c r="G220" t="n">
-        <v>10</v>
-      </c>
       <c r="H220" s="9" t="n"/>
       <c r="I220" s="9" t="n"/>
       <c r="K220" s="9" t="n"/>
     </row>
     <row r="221">
-      <c r="G221" t="n">
-        <v>10</v>
-      </c>
       <c r="H221" s="9" t="n"/>
       <c r="I221" s="9" t="n"/>
       <c r="K221" s="9" t="n"/>
     </row>
     <row r="222">
-      <c r="G222" t="n">
-        <v>10</v>
-      </c>
       <c r="H222" s="9" t="n"/>
       <c r="I222" s="9" t="n"/>
       <c r="K222" s="9" t="n"/>
     </row>
     <row r="223">
-      <c r="G223" t="n">
-        <v>10</v>
-      </c>
       <c r="H223" s="9" t="n"/>
       <c r="I223" s="9" t="n"/>
       <c r="K223" s="9" t="n"/>
     </row>
     <row r="224">
-      <c r="G224" t="n">
-        <v>10</v>
-      </c>
       <c r="H224" s="9" t="n"/>
       <c r="I224" s="9" t="n"/>
       <c r="K224" s="9" t="n"/>
     </row>
     <row r="225">
-      <c r="G225" t="n">
-        <v>10</v>
-      </c>
       <c r="H225" s="9" t="n"/>
       <c r="I225" s="9" t="n"/>
       <c r="K225" s="9" t="n"/>
     </row>
     <row r="226">
-      <c r="G226" t="n">
-        <v>10</v>
-      </c>
       <c r="H226" s="9" t="n"/>
       <c r="I226" s="9" t="n"/>
       <c r="K226" s="9" t="n"/>
     </row>
     <row r="227">
-      <c r="G227" t="n">
-        <v>10</v>
-      </c>
       <c r="H227" s="9" t="n"/>
       <c r="I227" s="9" t="n"/>
       <c r="K227" s="9" t="n"/>
     </row>
     <row r="228">
-      <c r="G228" t="n">
-        <v>10</v>
-      </c>
       <c r="H228" s="9" t="n"/>
       <c r="I228" s="9" t="n"/>
       <c r="K228" s="9" t="n"/>
     </row>
     <row r="229">
-      <c r="G229" t="n">
-        <v>10</v>
-      </c>
       <c r="H229" s="9" t="n"/>
       <c r="I229" s="9" t="n"/>
       <c r="K229" s="9" t="n"/>
     </row>
     <row r="230">
-      <c r="G230" t="n">
-        <v>10</v>
-      </c>
       <c r="H230" s="9" t="n"/>
       <c r="I230" s="9" t="n"/>
       <c r="K230" s="9" t="n"/>
     </row>
     <row r="231">
-      <c r="G231" t="n">
-        <v>10</v>
-      </c>
       <c r="H231" s="9" t="n"/>
       <c r="I231" s="9" t="n"/>
       <c r="K231" s="9" t="n"/>
     </row>
     <row r="232">
-      <c r="G232" t="n">
-        <v>10</v>
-      </c>
       <c r="H232" s="9" t="n"/>
       <c r="I232" s="9" t="n"/>
       <c r="K232" s="9" t="n"/>
     </row>
     <row r="233">
-      <c r="G233" t="n">
-        <v>10</v>
-      </c>
       <c r="H233" s="9" t="n"/>
       <c r="I233" s="9" t="n"/>
       <c r="K233" s="9" t="n"/>
     </row>
     <row r="234">
-      <c r="G234" t="n">
-        <v>10</v>
-      </c>
       <c r="H234" s="9" t="n"/>
       <c r="I234" s="9" t="n"/>
       <c r="K234" s="9" t="n"/>
     </row>
     <row r="235">
-      <c r="G235" t="n">
-        <v>10</v>
-      </c>
       <c r="H235" s="9" t="n"/>
       <c r="I235" s="9" t="n"/>
       <c r="K235" s="9" t="n"/>
     </row>
     <row r="236">
-      <c r="G236" t="n">
-        <v>10</v>
-      </c>
       <c r="H236" s="9" t="n"/>
       <c r="I236" s="9" t="n"/>
       <c r="K236" s="9" t="n"/>
     </row>
     <row r="237">
-      <c r="G237" t="n">
-        <v>10</v>
-      </c>
       <c r="H237" s="9" t="n"/>
       <c r="I237" s="9" t="n"/>
       <c r="K237" s="9" t="n"/>
     </row>
     <row r="238">
-      <c r="G238" t="n">
-        <v>10</v>
-      </c>
       <c r="H238" s="9" t="n"/>
       <c r="I238" s="9" t="n"/>
       <c r="K238" s="9" t="n"/>
     </row>
     <row r="239">
-      <c r="G239" t="n">
-        <v>10</v>
-      </c>
       <c r="H239" s="9" t="n"/>
       <c r="I239" s="9" t="n"/>
       <c r="K239" s="9" t="n"/>
     </row>
     <row r="240">
-      <c r="G240" t="n">
-        <v>10</v>
-      </c>
       <c r="H240" s="9" t="n"/>
       <c r="I240" s="9" t="n"/>
       <c r="K240" s="9" t="n"/>
     </row>
     <row r="241">
-      <c r="G241" t="n">
-        <v>10</v>
-      </c>
       <c r="H241" s="9" t="n"/>
       <c r="I241" s="9" t="n"/>
       <c r="K241" s="9" t="n"/>
     </row>
     <row r="242">
-      <c r="G242" t="n">
-        <v>10</v>
-      </c>
       <c r="H242" s="9" t="n"/>
       <c r="I242" s="9" t="n"/>
       <c r="K242" s="9" t="n"/>
     </row>
     <row r="243">
-      <c r="G243" t="n">
-        <v>10</v>
-      </c>
       <c r="H243" s="9" t="n"/>
       <c r="I243" s="9" t="n"/>
       <c r="K243" s="9" t="n"/>
     </row>
     <row r="244">
-      <c r="G244" t="n">
-        <v>10</v>
-      </c>
       <c r="H244" s="9" t="n"/>
       <c r="I244" s="9" t="n"/>
       <c r="K244" s="9" t="n"/>
     </row>
     <row r="245">
-      <c r="G245" t="n">
-        <v>10</v>
-      </c>
       <c r="H245" s="9" t="n"/>
       <c r="I245" s="9" t="n"/>
       <c r="K245" s="9" t="n"/>
     </row>
     <row r="246">
-      <c r="G246" t="n">
-        <v>10</v>
-      </c>
       <c r="H246" s="9" t="n"/>
       <c r="I246" s="9" t="n"/>
       <c r="K246" s="9" t="n"/>
     </row>
     <row r="247">
-      <c r="G247" t="n">
-        <v>10</v>
-      </c>
       <c r="H247" s="9" t="n"/>
       <c r="I247" s="9" t="n"/>
       <c r="K247" s="9" t="n"/>
     </row>
     <row r="248">
-      <c r="G248" t="n">
-        <v>10</v>
-      </c>
       <c r="H248" s="9" t="n"/>
       <c r="I248" s="9" t="n"/>
       <c r="K248" s="9" t="n"/>
     </row>
     <row r="249">
-      <c r="G249" t="n">
-        <v>10</v>
-      </c>
       <c r="H249" s="9" t="n"/>
       <c r="I249" s="9" t="n"/>
       <c r="K249" s="9" t="n"/>
     </row>
     <row r="250">
-      <c r="G250" t="n">
-        <v>10</v>
-      </c>
       <c r="H250" s="9" t="n"/>
       <c r="I250" s="9" t="n"/>
       <c r="K250" s="9" t="n"/>
     </row>
     <row r="251">
-      <c r="G251" t="n">
-        <v>10</v>
-      </c>
       <c r="H251" s="9" t="n"/>
       <c r="I251" s="9" t="n"/>
       <c r="K251" s="9" t="n"/>
     </row>
     <row r="252">
-      <c r="G252" t="n">
-        <v>10</v>
-      </c>
       <c r="H252" s="9" t="n"/>
       <c r="I252" s="9" t="n"/>
       <c r="K252" s="9" t="n"/>
     </row>
     <row r="253">
-      <c r="G253" t="n">
-        <v>10</v>
-      </c>
       <c r="H253" s="9" t="n"/>
       <c r="I253" s="9" t="n"/>
       <c r="K253" s="9" t="n"/>
     </row>
     <row r="254">
-      <c r="G254" t="n">
-        <v>10</v>
-      </c>
       <c r="H254" s="9" t="n"/>
       <c r="I254" s="9" t="n"/>
       <c r="K254" s="9" t="n"/>
     </row>
     <row r="255">
-      <c r="G255" t="n">
-        <v>10</v>
-      </c>
       <c r="H255" s="9" t="n"/>
       <c r="I255" s="9" t="n"/>
       <c r="K255" s="9" t="n"/>
     </row>
     <row r="256">
-      <c r="G256" t="n">
-        <v>10</v>
-      </c>
       <c r="H256" s="9" t="n"/>
       <c r="I256" s="9" t="n"/>
       <c r="K256" s="9" t="n"/>
     </row>
     <row r="257">
-      <c r="G257" t="n">
-        <v>10</v>
-      </c>
       <c r="H257" s="9" t="n"/>
       <c r="I257" s="9" t="n"/>
       <c r="K257" s="9" t="n"/>
     </row>
     <row r="258">
-      <c r="G258" t="n">
-        <v>10</v>
-      </c>
       <c r="H258" s="9" t="n"/>
       <c r="I258" s="9" t="n"/>
       <c r="K258" s="9" t="n"/>
     </row>
     <row r="259">
-      <c r="G259" t="n">
-        <v>10</v>
-      </c>
       <c r="H259" s="9" t="n"/>
       <c r="I259" s="9" t="n"/>
       <c r="K259" s="9" t="n"/>
     </row>
     <row r="260">
-      <c r="G260" t="n">
-        <v>10</v>
-      </c>
       <c r="H260" s="9" t="n"/>
       <c r="I260" s="9" t="n"/>
       <c r="K260" s="9" t="n"/>
     </row>
     <row r="261">
-      <c r="G261" t="n">
-        <v>10</v>
-      </c>
       <c r="H261" s="9" t="n"/>
       <c r="I261" s="9" t="n"/>
       <c r="K261" s="9" t="n"/>
     </row>
     <row r="262">
-      <c r="G262" t="n">
-        <v>10</v>
-      </c>
       <c r="H262" s="9" t="n"/>
       <c r="I262" s="9" t="n"/>
       <c r="K262" s="9" t="n"/>
     </row>
     <row r="263">
-      <c r="G263" t="n">
-        <v>10</v>
-      </c>
       <c r="H263" s="9" t="n"/>
       <c r="I263" s="9" t="n"/>
       <c r="K263" s="9" t="n"/>
     </row>
     <row r="264">
-      <c r="G264" t="n">
-        <v>10</v>
-      </c>
       <c r="H264" s="9" t="n"/>
       <c r="I264" s="9" t="n"/>
       <c r="K264" s="9" t="n"/>
     </row>
     <row r="265">
-      <c r="G265" t="n">
-        <v>10</v>
-      </c>
       <c r="H265" s="9" t="n"/>
       <c r="I265" s="9" t="n"/>
       <c r="K265" s="9" t="n"/>
     </row>
     <row r="266">
-      <c r="G266" t="n">
-        <v>10</v>
-      </c>
       <c r="H266" s="9" t="n"/>
       <c r="I266" s="9" t="n"/>
       <c r="K266" s="9" t="n"/>
     </row>
     <row r="267">
-      <c r="G267" t="n">
-        <v>10</v>
-      </c>
       <c r="H267" s="9" t="n"/>
       <c r="I267" s="9" t="n"/>
       <c r="K267" s="9" t="n"/>
     </row>
     <row r="268">
-      <c r="G268" t="n">
-        <v>10</v>
-      </c>
       <c r="H268" s="9" t="n"/>
       <c r="I268" s="9" t="n"/>
       <c r="K268" s="9" t="n"/>
     </row>
     <row r="269">
-      <c r="G269" t="n">
-        <v>10</v>
-      </c>
       <c r="H269" s="9" t="n"/>
       <c r="I269" s="9" t="n"/>
       <c r="K269" s="9" t="n"/>
     </row>
     <row r="270">
-      <c r="G270" t="n">
-        <v>10</v>
-      </c>
       <c r="H270" s="9" t="n"/>
       <c r="I270" s="9" t="n"/>
       <c r="K270" s="9" t="n"/>
     </row>
     <row r="271">
-      <c r="G271" t="n">
-        <v>10</v>
-      </c>
       <c r="H271" s="9" t="n"/>
       <c r="I271" s="9" t="n"/>
       <c r="K271" s="9" t="n"/>
     </row>
     <row r="272">
-      <c r="G272" t="n">
-        <v>10</v>
-      </c>
       <c r="H272" s="9" t="n"/>
       <c r="I272" s="9" t="n"/>
       <c r="K272" s="9" t="n"/>
     </row>
     <row r="273">
-      <c r="G273" t="n">
-        <v>10</v>
-      </c>
       <c r="H273" s="9" t="n"/>
       <c r="I273" s="9" t="n"/>
       <c r="K273" s="9" t="n"/>
     </row>
     <row r="274">
-      <c r="G274" t="n">
-        <v>10</v>
-      </c>
       <c r="H274" s="9" t="n"/>
       <c r="I274" s="9" t="n"/>
       <c r="K274" s="9" t="n"/>
     </row>
     <row r="275">
-      <c r="G275" t="n">
-        <v>10</v>
-      </c>
       <c r="H275" s="9" t="n"/>
       <c r="I275" s="9" t="n"/>
       <c r="K275" s="9" t="n"/>
     </row>
     <row r="276">
-      <c r="G276" t="n">
-        <v>10</v>
-      </c>
       <c r="H276" s="9" t="n"/>
       <c r="I276" s="9" t="n"/>
       <c r="K276" s="9" t="n"/>
     </row>
     <row r="277">
-      <c r="G277" t="n">
-        <v>10</v>
-      </c>
       <c r="H277" s="9" t="n"/>
       <c r="I277" s="9" t="n"/>
       <c r="K277" s="9" t="n"/>
     </row>
     <row r="278">
-      <c r="G278" t="n">
-        <v>10</v>
-      </c>
       <c r="H278" s="9" t="n"/>
       <c r="I278" s="9" t="n"/>
       <c r="K278" s="9" t="n"/>
     </row>
     <row r="279">
-      <c r="G279" t="n">
-        <v>10</v>
-      </c>
       <c r="H279" s="9" t="n"/>
       <c r="I279" s="9" t="n"/>
       <c r="K279" s="9" t="n"/>
     </row>
     <row r="280">
-      <c r="G280" t="n">
-        <v>10</v>
-      </c>
       <c r="H280" s="9" t="n"/>
       <c r="I280" s="9" t="n"/>
       <c r="K280" s="9" t="n"/>
     </row>
     <row r="281">
-      <c r="G281" t="n">
-        <v>10</v>
-      </c>
       <c r="H281" s="9" t="n"/>
       <c r="I281" s="9" t="n"/>
       <c r="K281" s="9" t="n"/>
     </row>
     <row r="282">
-      <c r="G282" t="n">
-        <v>10</v>
-      </c>
       <c r="H282" s="9" t="n"/>
       <c r="I282" s="9" t="n"/>
       <c r="K282" s="9" t="n"/>
     </row>
     <row r="283">
-      <c r="G283" t="n">
-        <v>10</v>
-      </c>
       <c r="H283" s="9" t="n"/>
       <c r="I283" s="9" t="n"/>
       <c r="K283" s="9" t="n"/>
     </row>
     <row r="284">
-      <c r="G284" t="n">
-        <v>10</v>
-      </c>
       <c r="H284" s="9" t="n"/>
       <c r="I284" s="9" t="n"/>
       <c r="K284" s="9" t="n"/>
     </row>
     <row r="285">
-      <c r="G285" t="n">
-        <v>10</v>
-      </c>
       <c r="H285" s="9" t="n"/>
       <c r="I285" s="9" t="n"/>
       <c r="K285" s="9" t="n"/>
     </row>
     <row r="286">
-      <c r="G286" t="n">
-        <v>10</v>
-      </c>
       <c r="H286" s="9" t="n"/>
       <c r="I286" s="9" t="n"/>
       <c r="K286" s="9" t="n"/>
     </row>
     <row r="287">
-      <c r="G287" t="n">
-        <v>10</v>
-      </c>
       <c r="H287" s="9" t="n"/>
       <c r="I287" s="9" t="n"/>
       <c r="K287" s="9" t="n"/>
     </row>
     <row r="288">
-      <c r="G288" t="n">
-        <v>10</v>
-      </c>
       <c r="H288" s="9" t="n"/>
       <c r="I288" s="9" t="n"/>
       <c r="K288" s="9" t="n"/>
     </row>
     <row r="289">
-      <c r="G289" t="n">
-        <v>10</v>
-      </c>
       <c r="H289" s="9" t="n"/>
       <c r="I289" s="9" t="n"/>
       <c r="K289" s="9" t="n"/>
     </row>
     <row r="290">
-      <c r="G290" t="n">
-        <v>10</v>
-      </c>
       <c r="H290" s="9" t="n"/>
       <c r="I290" s="9" t="n"/>
       <c r="K290" s="9" t="n"/>
     </row>
     <row r="291">
-      <c r="G291" t="n">
-        <v>10</v>
-      </c>
       <c r="H291" s="9" t="n"/>
       <c r="I291" s="9" t="n"/>
       <c r="K291" s="9" t="n"/>
     </row>
     <row r="292">
-      <c r="G292" t="n">
-        <v>10</v>
-      </c>
       <c r="H292" s="9" t="n"/>
       <c r="I292" s="9" t="n"/>
       <c r="K292" s="9" t="n"/>
     </row>
     <row r="293">
-      <c r="G293" t="n">
-        <v>10</v>
-      </c>
       <c r="H293" s="9" t="n"/>
       <c r="I293" s="9" t="n"/>
       <c r="K293" s="9" t="n"/>
     </row>
     <row r="294">
-      <c r="G294" t="n">
-        <v>10</v>
-      </c>
       <c r="H294" s="9" t="n"/>
       <c r="I294" s="9" t="n"/>
       <c r="K294" s="9" t="n"/>
     </row>
     <row r="295">
-      <c r="G295" t="n">
-        <v>10</v>
-      </c>
       <c r="H295" s="9" t="n"/>
       <c r="I295" s="9" t="n"/>
       <c r="K295" s="9" t="n"/>
     </row>
     <row r="296">
-      <c r="G296" t="n">
-        <v>10</v>
-      </c>
       <c r="H296" s="9" t="n"/>
       <c r="I296" s="9" t="n"/>
       <c r="K296" s="9" t="n"/>
     </row>
     <row r="297">
-      <c r="G297" t="n">
-        <v>10</v>
-      </c>
       <c r="H297" s="9" t="n"/>
       <c r="I297" s="9" t="n"/>
       <c r="K297" s="9" t="n"/>
     </row>
     <row r="298">
-      <c r="G298" t="n">
-        <v>10</v>
-      </c>
       <c r="H298" s="9" t="n"/>
       <c r="I298" s="9" t="n"/>
       <c r="K298" s="9" t="n"/>
     </row>
     <row r="299">
-      <c r="G299" t="n">
-        <v>10</v>
-      </c>
       <c r="H299" s="9" t="n"/>
       <c r="I299" s="9" t="n"/>
       <c r="K299" s="9" t="n"/>
     </row>
     <row r="300">
-      <c r="G300" t="n">
-        <v>10</v>
-      </c>
       <c r="H300" s="9" t="n"/>
       <c r="I300" s="9" t="n"/>
       <c r="K300" s="9" t="n"/>
     </row>
     <row r="301">
-      <c r="G301" t="n">
-        <v>10</v>
-      </c>
       <c r="H301" s="9" t="n"/>
       <c r="I301" s="9" t="n"/>
       <c r="K301" s="9" t="n"/>
     </row>
     <row r="302">
-      <c r="G302" t="n">
-        <v>10</v>
-      </c>
       <c r="H302" s="9" t="n"/>
       <c r="I302" s="9" t="n"/>
       <c r="K302" s="9" t="n"/>
     </row>
     <row r="303">
-      <c r="G303" t="n">
-        <v>10</v>
-      </c>
       <c r="H303" s="9" t="n"/>
       <c r="I303" s="9" t="n"/>
       <c r="K303" s="9" t="n"/>
     </row>
     <row r="304">
-      <c r="G304" t="n">
-        <v>10</v>
-      </c>
       <c r="H304" s="9" t="n"/>
       <c r="I304" s="9" t="n"/>
       <c r="K304" s="9" t="n"/>
     </row>
     <row r="305">
-      <c r="G305" t="n">
-        <v>10</v>
-      </c>
       <c r="H305" s="9" t="n"/>
       <c r="I305" s="9" t="n"/>
       <c r="K305" s="9" t="n"/>
     </row>
     <row r="306">
-      <c r="G306" t="n">
-        <v>10</v>
-      </c>
       <c r="H306" s="9" t="n"/>
       <c r="I306" s="9" t="n"/>
       <c r="K306" s="9" t="n"/>
     </row>
     <row r="307">
-      <c r="G307" t="n">
-        <v>10</v>
-      </c>
       <c r="H307" s="9" t="n"/>
       <c r="I307" s="9" t="n"/>
       <c r="K307" s="9" t="n"/>
     </row>
     <row r="308">
-      <c r="G308" t="n">
-        <v>10</v>
-      </c>
       <c r="H308" s="9" t="n"/>
       <c r="I308" s="9" t="n"/>
       <c r="K308" s="9" t="n"/>
     </row>
     <row r="309">
-      <c r="G309" t="n">
-        <v>10</v>
-      </c>
       <c r="H309" s="9" t="n"/>
       <c r="I309" s="9" t="n"/>
       <c r="K309" s="9" t="n"/>
     </row>
     <row r="310">
-      <c r="G310" t="n">
-        <v>10</v>
-      </c>
       <c r="H310" s="9" t="n"/>
       <c r="I310" s="9" t="n"/>
       <c r="K310" s="9" t="n"/>
     </row>
     <row r="311">
-      <c r="G311" t="n">
-        <v>10</v>
-      </c>
       <c r="H311" s="9" t="n"/>
       <c r="I311" s="9" t="n"/>
       <c r="K311" s="9" t="n"/>
     </row>
     <row r="312">
-      <c r="G312" t="n">
-        <v>10</v>
-      </c>
       <c r="H312" s="9" t="n"/>
       <c r="I312" s="9" t="n"/>
       <c r="K312" s="9" t="n"/>
     </row>
     <row r="313">
-      <c r="G313" t="n">
-        <v>10</v>
-      </c>
       <c r="H313" s="9" t="n"/>
       <c r="I313" s="9" t="n"/>
       <c r="K313" s="9" t="n"/>
     </row>
     <row r="314">
-      <c r="G314" t="n">
-        <v>10</v>
-      </c>
       <c r="H314" s="9" t="n"/>
       <c r="I314" s="9" t="n"/>
       <c r="K314" s="9" t="n"/>
     </row>
     <row r="315">
-      <c r="G315" t="n">
-        <v>10</v>
-      </c>
       <c r="H315" s="9" t="n"/>
       <c r="I315" s="9" t="n"/>
       <c r="K315" s="9" t="n"/>
     </row>
     <row r="316">
-      <c r="G316" t="n">
-        <v>10</v>
-      </c>
       <c r="H316" s="9" t="n"/>
       <c r="I316" s="9" t="n"/>
       <c r="K316" s="9" t="n"/>
     </row>
     <row r="317">
-      <c r="G317" t="n">
-        <v>10</v>
-      </c>
       <c r="H317" s="9" t="n"/>
       <c r="I317" s="9" t="n"/>
       <c r="K317" s="9" t="n"/>
     </row>
     <row r="318">
-      <c r="G318" t="n">
-        <v>10</v>
-      </c>
       <c r="H318" s="9" t="n"/>
       <c r="I318" s="9" t="n"/>
       <c r="K318" s="9" t="n"/>
     </row>
     <row r="319">
-      <c r="G319" t="n">
-        <v>10</v>
-      </c>
       <c r="H319" s="9" t="n"/>
       <c r="I319" s="9" t="n"/>
       <c r="K319" s="9" t="n"/>
     </row>
     <row r="320">
-      <c r="G320" t="n">
-        <v>10</v>
-      </c>
       <c r="H320" s="9" t="n"/>
       <c r="I320" s="9" t="n"/>
       <c r="K320" s="9" t="n"/>
     </row>
     <row r="321">
-      <c r="G321" t="n">
-        <v>10</v>
-      </c>
       <c r="H321" s="9" t="n"/>
       <c r="I321" s="9" t="n"/>
       <c r="K321" s="9" t="n"/>
     </row>
     <row r="322">
-      <c r="G322" t="n">
-        <v>10</v>
-      </c>
       <c r="H322" s="9" t="n"/>
       <c r="I322" s="9" t="n"/>
       <c r="K322" s="9" t="n"/>
     </row>
     <row r="323">
-      <c r="G323" t="n">
-        <v>10</v>
-      </c>
       <c r="H323" s="9" t="n"/>
       <c r="I323" s="9" t="n"/>
       <c r="K323" s="9" t="n"/>
     </row>
     <row r="324">
-      <c r="G324" t="n">
-        <v>10</v>
-      </c>
       <c r="H324" s="9" t="n"/>
       <c r="I324" s="9" t="n"/>
       <c r="K324" s="9" t="n"/>
     </row>
     <row r="325">
-      <c r="G325" t="n">
-        <v>10</v>
-      </c>
       <c r="H325" s="9" t="n"/>
       <c r="I325" s="9" t="n"/>
       <c r="K325" s="9" t="n"/>
     </row>
     <row r="326">
-      <c r="G326" t="n">
-        <v>10</v>
-      </c>
       <c r="H326" s="9" t="n"/>
       <c r="I326" s="9" t="n"/>
       <c r="K326" s="9" t="n"/>
     </row>
     <row r="327">
-      <c r="G327" t="n">
-        <v>10</v>
-      </c>
       <c r="H327" s="9" t="n"/>
       <c r="I327" s="9" t="n"/>
       <c r="K327" s="9" t="n"/>
     </row>
     <row r="328">
-      <c r="G328" t="n">
-        <v>10</v>
-      </c>
       <c r="H328" s="9" t="n"/>
       <c r="I328" s="9" t="n"/>
       <c r="K328" s="9" t="n"/>
     </row>
     <row r="329">
-      <c r="G329" t="n">
-        <v>10</v>
-      </c>
       <c r="H329" s="9" t="n"/>
       <c r="I329" s="9" t="n"/>
       <c r="K329" s="9" t="n"/>
     </row>
     <row r="330">
-      <c r="G330" t="n">
-        <v>10</v>
-      </c>
       <c r="H330" s="9" t="n"/>
       <c r="I330" s="9" t="n"/>
       <c r="K330" s="9" t="n"/>
     </row>
     <row r="331">
-      <c r="G331" t="n">
-        <v>10</v>
-      </c>
       <c r="H331" s="9" t="n"/>
       <c r="I331" s="9" t="n"/>
       <c r="K331" s="9" t="n"/>
     </row>
     <row r="332">
-      <c r="G332" t="n">
-        <v>10</v>
-      </c>
       <c r="H332" s="9" t="n"/>
       <c r="I332" s="9" t="n"/>
       <c r="K332" s="9" t="n"/>
     </row>
     <row r="333">
-      <c r="G333" t="n">
-        <v>10</v>
-      </c>
       <c r="H333" s="9" t="n"/>
       <c r="I333" s="9" t="n"/>
       <c r="K333" s="9" t="n"/>
     </row>
     <row r="334">
-      <c r="G334" t="n">
-        <v>10</v>
-      </c>
       <c r="H334" s="9" t="n"/>
       <c r="I334" s="9" t="n"/>
       <c r="K334" s="9" t="n"/>
     </row>
     <row r="335">
-      <c r="G335" t="n">
-        <v>10</v>
-      </c>
       <c r="H335" s="9" t="n"/>
       <c r="I335" s="9" t="n"/>
       <c r="K335" s="9" t="n"/>
     </row>
     <row r="336">
-      <c r="G336" t="n">
-        <v>10</v>
-      </c>
       <c r="H336" s="9" t="n"/>
       <c r="I336" s="9" t="n"/>
       <c r="K336" s="9" t="n"/>
     </row>
     <row r="337">
-      <c r="G337" t="n">
-        <v>10</v>
-      </c>
       <c r="H337" s="9" t="n"/>
       <c r="I337" s="9" t="n"/>
       <c r="K337" s="9" t="n"/>
     </row>
     <row r="338">
-      <c r="G338" t="n">
-        <v>10</v>
-      </c>
       <c r="H338" s="9" t="n"/>
       <c r="I338" s="9" t="n"/>
       <c r="K338" s="9" t="n"/>
     </row>
     <row r="339">
-      <c r="G339" t="n">
-        <v>10</v>
-      </c>
       <c r="H339" s="9" t="n"/>
       <c r="I339" s="9" t="n"/>
       <c r="K339" s="9" t="n"/>
     </row>
     <row r="340">
-      <c r="G340" t="n">
-        <v>10</v>
-      </c>
       <c r="H340" s="9" t="n"/>
       <c r="I340" s="9" t="n"/>
       <c r="K340" s="9" t="n"/>
     </row>
     <row r="341">
-      <c r="G341" t="n">
-        <v>10</v>
-      </c>
       <c r="H341" s="9" t="n"/>
       <c r="I341" s="9" t="n"/>
       <c r="K341" s="9" t="n"/>
     </row>
     <row r="342">
-      <c r="G342" t="n">
-        <v>10</v>
-      </c>
       <c r="H342" s="9" t="n"/>
       <c r="I342" s="9" t="n"/>
       <c r="K342" s="9" t="n"/>
     </row>
     <row r="343">
-      <c r="G343" t="n">
-        <v>10</v>
-      </c>
       <c r="H343" s="9" t="n"/>
       <c r="I343" s="9" t="n"/>
       <c r="K343" s="9" t="n"/>
     </row>
     <row r="344">
-      <c r="G344" t="n">
-        <v>10</v>
-      </c>
       <c r="H344" s="9" t="n"/>
       <c r="I344" s="9" t="n"/>
       <c r="K344" s="9" t="n"/>
     </row>
     <row r="345">
-      <c r="G345" t="n">
-        <v>10</v>
-      </c>
       <c r="H345" s="9" t="n"/>
       <c r="I345" s="9" t="n"/>
       <c r="K345" s="9" t="n"/>
     </row>
     <row r="346">
-      <c r="G346" t="n">
-        <v>10</v>
-      </c>
       <c r="H346" s="9" t="n"/>
       <c r="I346" s="9" t="n"/>
       <c r="K346" s="9" t="n"/>
     </row>
     <row r="347">
-      <c r="G347" t="n">
-        <v>10</v>
-      </c>
       <c r="H347" s="9" t="n"/>
       <c r="I347" s="9" t="n"/>
       <c r="K347" s="9" t="n"/>
     </row>
     <row r="348">
-      <c r="G348" t="n">
-        <v>10</v>
-      </c>
       <c r="H348" s="9" t="n"/>
       <c r="I348" s="9" t="n"/>
       <c r="K348" s="9" t="n"/>
     </row>
     <row r="349">
-      <c r="G349" t="n">
-        <v>10</v>
-      </c>
       <c r="H349" s="9" t="n"/>
       <c r="I349" s="9" t="n"/>
       <c r="K349" s="9" t="n"/>
     </row>
     <row r="350">
-      <c r="G350" t="n">
-        <v>10</v>
-      </c>
       <c r="H350" s="9" t="n"/>
       <c r="I350" s="9" t="n"/>
       <c r="K350" s="9" t="n"/>
     </row>
     <row r="351">
-      <c r="G351" t="n">
-        <v>10</v>
-      </c>
       <c r="H351" s="9" t="n"/>
       <c r="I351" s="9" t="n"/>
       <c r="K351" s="9" t="n"/>
     </row>
     <row r="352">
-      <c r="G352" t="n">
-        <v>10</v>
-      </c>
       <c r="H352" s="9" t="n"/>
       <c r="I352" s="9" t="n"/>
       <c r="K352" s="9" t="n"/>
     </row>
     <row r="353">
-      <c r="G353" t="n">
-        <v>10</v>
-      </c>
       <c r="H353" s="9" t="n"/>
       <c r="I353" s="9" t="n"/>
       <c r="K353" s="9" t="n"/>
     </row>
     <row r="354">
-      <c r="G354" t="n">
-        <v>10</v>
-      </c>
       <c r="H354" s="9" t="n"/>
       <c r="I354" s="9" t="n"/>
       <c r="K354" s="9" t="n"/>
     </row>
     <row r="355">
-      <c r="G355" t="n">
-        <v>10</v>
-      </c>
       <c r="H355" s="9" t="n"/>
       <c r="I355" s="9" t="n"/>
       <c r="K355" s="9" t="n"/>
     </row>
     <row r="356">
-      <c r="G356" t="n">
-        <v>10</v>
-      </c>
       <c r="H356" s="9" t="n"/>
       <c r="I356" s="9" t="n"/>
       <c r="K356" s="9" t="n"/>
     </row>
     <row r="357">
-      <c r="G357" t="n">
-        <v>10</v>
-      </c>
       <c r="H357" s="9" t="n"/>
       <c r="I357" s="9" t="n"/>
       <c r="K357" s="9" t="n"/>
     </row>
     <row r="358">
-      <c r="G358" t="n">
-        <v>10</v>
-      </c>
       <c r="H358" s="9" t="n"/>
       <c r="I358" s="9" t="n"/>
       <c r="K358" s="9" t="n"/>
     </row>
     <row r="359">
-      <c r="G359" t="n">
-        <v>10</v>
-      </c>
       <c r="H359" s="9" t="n"/>
       <c r="I359" s="9" t="n"/>
       <c r="K359" s="9" t="n"/>
     </row>
     <row r="360">
-      <c r="G360" t="n">
-        <v>10</v>
-      </c>
       <c r="H360" s="9" t="n"/>
       <c r="I360" s="9" t="n"/>
       <c r="K360" s="9" t="n"/>
     </row>
     <row r="361">
-      <c r="G361" t="n">
-        <v>10</v>
-      </c>
       <c r="H361" s="9" t="n"/>
       <c r="I361" s="9" t="n"/>
       <c r="K361" s="9" t="n"/>
     </row>
     <row r="362">
-      <c r="G362" t="n">
-        <v>10</v>
-      </c>
       <c r="H362" s="9" t="n"/>
       <c r="I362" s="9" t="n"/>
       <c r="K362" s="9" t="n"/>
     </row>
     <row r="363">
-      <c r="G363" t="n">
-        <v>10</v>
-      </c>
       <c r="H363" s="9" t="n"/>
       <c r="I363" s="9" t="n"/>
       <c r="K363" s="9" t="n"/>
     </row>
     <row r="364">
-      <c r="G364" t="n">
-        <v>10</v>
-      </c>
       <c r="H364" s="9" t="n"/>
       <c r="I364" s="9" t="n"/>
       <c r="K364" s="9" t="n"/>
     </row>
     <row r="365">
-      <c r="G365" t="n">
-        <v>10</v>
-      </c>
       <c r="H365" s="9" t="n"/>
       <c r="I365" s="9" t="n"/>
       <c r="K365" s="9" t="n"/>
     </row>
     <row r="366">
-      <c r="G366" t="n">
-        <v>10</v>
-      </c>
       <c r="H366" s="9" t="n"/>
       <c r="I366" s="9" t="n"/>
       <c r="K366" s="9" t="n"/>
     </row>
     <row r="367">
-      <c r="G367" t="n">
-        <v>10</v>
-      </c>
       <c r="H367" s="9" t="n"/>
       <c r="I367" s="9" t="n"/>
       <c r="K367" s="9" t="n"/>
     </row>
     <row r="368">
-      <c r="G368" t="n">
-        <v>10</v>
-      </c>
       <c r="H368" s="9" t="n"/>
       <c r="I368" s="9" t="n"/>
       <c r="K368" s="9" t="n"/>
     </row>
     <row r="369">
-      <c r="G369" t="n">
-        <v>10</v>
-      </c>
       <c r="H369" s="9" t="n"/>
       <c r="I369" s="9" t="n"/>
       <c r="K369" s="9" t="n"/>
     </row>
     <row r="370">
-      <c r="G370" t="n">
-        <v>10</v>
-      </c>
       <c r="H370" s="9" t="n"/>
       <c r="I370" s="9" t="n"/>
       <c r="K370" s="9" t="n"/>
     </row>
     <row r="371">
-      <c r="G371" t="n">
-        <v>10</v>
-      </c>
       <c r="H371" s="9" t="n"/>
       <c r="I371" s="9" t="n"/>
       <c r="K371" s="9" t="n"/>
     </row>
     <row r="372">
-      <c r="G372" t="n">
-        <v>10</v>
-      </c>
       <c r="H372" s="9" t="n"/>
       <c r="I372" s="9" t="n"/>
       <c r="K372" s="9" t="n"/>
     </row>
     <row r="373">
-      <c r="G373" t="n">
-        <v>10</v>
-      </c>
       <c r="H373" s="9" t="n"/>
       <c r="I373" s="9" t="n"/>
       <c r="K373" s="9" t="n"/>
     </row>
     <row r="374">
-      <c r="G374" t="n">
-        <v>10</v>
-      </c>
       <c r="H374" s="9" t="n"/>
       <c r="I374" s="9" t="n"/>
       <c r="K374" s="9" t="n"/>
     </row>
     <row r="375">
-      <c r="G375" t="n">
-        <v>10</v>
-      </c>
       <c r="H375" s="9" t="n"/>
       <c r="I375" s="9" t="n"/>
       <c r="K375" s="9" t="n"/>
     </row>
     <row r="376">
-      <c r="G376" t="n">
-        <v>10</v>
-      </c>
       <c r="H376" s="9" t="n"/>
       <c r="I376" s="9" t="n"/>
       <c r="K376" s="9" t="n"/>
     </row>
     <row r="377">
-      <c r="G377" t="n">
-        <v>10</v>
-      </c>
       <c r="H377" s="9" t="n"/>
       <c r="I377" s="9" t="n"/>
       <c r="K377" s="9" t="n"/>
     </row>
     <row r="378">
-      <c r="G378" t="n">
-        <v>10</v>
-      </c>
       <c r="H378" s="9" t="n"/>
       <c r="I378" s="9" t="n"/>
       <c r="K378" s="9" t="n"/>
     </row>
     <row r="379">
-      <c r="G379" t="n">
-        <v>10</v>
-      </c>
       <c r="H379" s="9" t="n"/>
       <c r="I379" s="9" t="n"/>
       <c r="K379" s="9" t="n"/>
     </row>
     <row r="380">
-      <c r="G380" t="n">
-        <v>10</v>
-      </c>
       <c r="H380" s="9" t="n"/>
       <c r="I380" s="9" t="n"/>
       <c r="K380" s="9" t="n"/>
     </row>
     <row r="381">
-      <c r="G381" t="n">
-        <v>10</v>
-      </c>
       <c r="H381" s="9" t="n"/>
       <c r="I381" s="9" t="n"/>
       <c r="K381" s="9" t="n"/>
     </row>
     <row r="382">
-      <c r="G382" t="n">
-        <v>10</v>
-      </c>
       <c r="H382" s="9" t="n"/>
       <c r="I382" s="9" t="n"/>
       <c r="K382" s="9" t="n"/>
     </row>
     <row r="383">
-      <c r="G383" t="n">
-        <v>10</v>
-      </c>
       <c r="H383" s="9" t="n"/>
       <c r="I383" s="9" t="n"/>
       <c r="K383" s="9" t="n"/>
     </row>
     <row r="384">
-      <c r="G384" t="n">
-        <v>10</v>
-      </c>
       <c r="H384" s="9" t="n"/>
       <c r="I384" s="9" t="n"/>
       <c r="K384" s="9" t="n"/>
     </row>
     <row r="385">
-      <c r="G385" t="n">
-        <v>10</v>
-      </c>
       <c r="H385" s="9" t="n"/>
       <c r="I385" s="9" t="n"/>
       <c r="K385" s="9" t="n"/>
     </row>
     <row r="386">
-      <c r="G386" t="n">
-        <v>10</v>
-      </c>
       <c r="H386" s="9" t="n"/>
       <c r="I386" s="9" t="n"/>
       <c r="K386" s="9" t="n"/>
     </row>
     <row r="387">
-      <c r="G387" t="n">
-        <v>10</v>
-      </c>
       <c r="H387" s="9" t="n"/>
       <c r="I387" s="9" t="n"/>
       <c r="K387" s="9" t="n"/>
     </row>
     <row r="388">
-      <c r="G388" t="n">
-        <v>10</v>
-      </c>
       <c r="H388" s="9" t="n"/>
       <c r="I388" s="9" t="n"/>
       <c r="K388" s="9" t="n"/>
     </row>
     <row r="389">
-      <c r="G389" t="n">
-        <v>10</v>
-      </c>
       <c r="H389" s="9" t="n"/>
       <c r="I389" s="9" t="n"/>
       <c r="K389" s="9" t="n"/>
     </row>
     <row r="390">
-      <c r="G390" t="n">
-        <v>10</v>
-      </c>
       <c r="H390" s="9" t="n"/>
       <c r="I390" s="9" t="n"/>
       <c r="K390" s="9" t="n"/>
     </row>
     <row r="391">
-      <c r="G391" t="n">
-        <v>10</v>
-      </c>
       <c r="H391" s="9" t="n"/>
       <c r="I391" s="9" t="n"/>
       <c r="K391" s="9" t="n"/>
     </row>
     <row r="392">
-      <c r="G392" t="n">
-        <v>10</v>
-      </c>
       <c r="H392" s="9" t="n"/>
       <c r="I392" s="9" t="n"/>
       <c r="K392" s="9" t="n"/>
     </row>
     <row r="393">
-      <c r="G393" t="n">
-        <v>10</v>
-      </c>
       <c r="H393" s="9" t="n"/>
       <c r="I393" s="9" t="n"/>
       <c r="K393" s="9" t="n"/>
     </row>
     <row r="394">
-      <c r="G394" t="n">
-        <v>10</v>
-      </c>
       <c r="H394" s="9" t="n"/>
       <c r="I394" s="9" t="n"/>
       <c r="K394" s="9" t="n"/>
     </row>
     <row r="395">
-      <c r="G395" t="n">
-        <v>10</v>
-      </c>
       <c r="H395" s="9" t="n"/>
       <c r="I395" s="9" t="n"/>
       <c r="K395" s="9" t="n"/>
     </row>
     <row r="396">
-      <c r="G396" t="n">
-        <v>10</v>
-      </c>
       <c r="H396" s="9" t="n"/>
       <c r="I396" s="9" t="n"/>
       <c r="K396" s="9" t="n"/>
     </row>
     <row r="397">
-      <c r="G397" t="n">
-        <v>10</v>
-      </c>
       <c r="H397" s="9" t="n"/>
       <c r="I397" s="9" t="n"/>
       <c r="K397" s="9" t="n"/>
     </row>
     <row r="398">
-      <c r="G398" t="n">
-        <v>10</v>
-      </c>
       <c r="H398" s="9" t="n"/>
       <c r="I398" s="9" t="n"/>
       <c r="K398" s="9" t="n"/>
     </row>
     <row r="399">
-      <c r="G399" t="n">
-        <v>10</v>
-      </c>
       <c r="H399" s="9" t="n"/>
       <c r="I399" s="9" t="n"/>
       <c r="K399" s="9" t="n"/>
     </row>
     <row r="400">
-      <c r="G400" t="n">
-        <v>10</v>
-      </c>
       <c r="H400" s="9" t="n"/>
       <c r="I400" s="9" t="n"/>
       <c r="K400" s="9" t="n"/>
     </row>
     <row r="401">
-      <c r="G401" t="n">
-        <v>10</v>
-      </c>
       <c r="H401" s="9" t="n"/>
       <c r="I401" s="9" t="n"/>
       <c r="K401" s="9" t="n"/>
     </row>
     <row r="402">
-      <c r="G402" t="n">
-        <v>10</v>
-      </c>
       <c r="H402" s="9" t="n"/>
       <c r="I402" s="9" t="n"/>
       <c r="K402" s="9" t="n"/>
     </row>
     <row r="403">
-      <c r="G403" t="n">
-        <v>10</v>
-      </c>
       <c r="H403" s="9" t="n"/>
       <c r="I403" s="9" t="n"/>
       <c r="K403" s="9" t="n"/>
     </row>
     <row r="404">
-      <c r="G404" t="n">
-        <v>10</v>
-      </c>
       <c r="H404" s="9" t="n"/>
       <c r="I404" s="9" t="n"/>
       <c r="K404" s="9" t="n"/>
     </row>
     <row r="405">
-      <c r="G405" t="n">
-        <v>10</v>
-      </c>
       <c r="H405" s="9" t="n"/>
       <c r="I405" s="9" t="n"/>
       <c r="K405" s="9" t="n"/>
     </row>
     <row r="406">
-      <c r="G406" t="n">
-        <v>10</v>
-      </c>
       <c r="H406" s="9" t="n"/>
       <c r="I406" s="9" t="n"/>
       <c r="K406" s="9" t="n"/>
     </row>
     <row r="407">
-      <c r="G407" t="n">
-        <v>10</v>
-      </c>
       <c r="H407" s="9" t="n"/>
       <c r="I407" s="9" t="n"/>
       <c r="K407" s="9" t="n"/>
     </row>
     <row r="408">
-      <c r="G408" t="n">
-        <v>10</v>
-      </c>
       <c r="H408" s="9" t="n"/>
       <c r="I408" s="9" t="n"/>
       <c r="K408" s="9" t="n"/>
     </row>
     <row r="409">
-      <c r="G409" t="n">
-        <v>10</v>
-      </c>
       <c r="H409" s="9" t="n"/>
       <c r="I409" s="9" t="n"/>
       <c r="K409" s="9" t="n"/>
     </row>
     <row r="410">
-      <c r="G410" t="n">
-        <v>10</v>
-      </c>
       <c r="H410" s="9" t="n"/>
       <c r="I410" s="9" t="n"/>
       <c r="K410" s="9" t="n"/>
     </row>
     <row r="411">
-      <c r="G411" t="n">
-        <v>10</v>
-      </c>
       <c r="H411" s="9" t="n"/>
       <c r="I411" s="9" t="n"/>
       <c r="K411" s="9" t="n"/>
     </row>
     <row r="412">
-      <c r="G412" t="n">
-        <v>10</v>
-      </c>
       <c r="H412" s="9" t="n"/>
       <c r="I412" s="9" t="n"/>
       <c r="K412" s="9" t="n"/>
     </row>
     <row r="413">
-      <c r="G413" t="n">
-        <v>10</v>
-      </c>
       <c r="H413" s="9" t="n"/>
       <c r="I413" s="9" t="n"/>
       <c r="K413" s="9" t="n"/>
     </row>
     <row r="414">
-      <c r="G414" t="n">
-        <v>10</v>
-      </c>
       <c r="H414" s="9" t="n"/>
       <c r="I414" s="9" t="n"/>
       <c r="K414" s="9" t="n"/>
     </row>
     <row r="415">
-      <c r="G415" t="n">
-        <v>10</v>
-      </c>
       <c r="H415" s="9" t="n"/>
       <c r="I415" s="9" t="n"/>
       <c r="K415" s="9" t="n"/>
     </row>
     <row r="416">
-      <c r="G416" t="n">
-        <v>10</v>
-      </c>
       <c r="H416" s="9" t="n"/>
       <c r="I416" s="9" t="n"/>
       <c r="K416" s="9" t="n"/>
     </row>
     <row r="417">
-      <c r="G417" t="n">
-        <v>10</v>
-      </c>
       <c r="H417" s="9" t="n"/>
       <c r="I417" s="9" t="n"/>
       <c r="K417" s="9" t="n"/>
     </row>
     <row r="418">
-      <c r="G418" t="n">
-        <v>10</v>
-      </c>
       <c r="H418" s="9" t="n"/>
       <c r="I418" s="9" t="n"/>
       <c r="K418" s="9" t="n"/>
     </row>
     <row r="419">
-      <c r="G419" t="n">
-        <v>10</v>
-      </c>
       <c r="H419" s="9" t="n"/>
       <c r="I419" s="9" t="n"/>
       <c r="K419" s="9" t="n"/>
     </row>
     <row r="420">
-      <c r="G420" t="n">
-        <v>10</v>
-      </c>
       <c r="H420" s="9" t="n"/>
       <c r="I420" s="9" t="n"/>
       <c r="K420" s="9" t="n"/>
     </row>
     <row r="421">
-      <c r="G421" t="n">
-        <v>10</v>
-      </c>
       <c r="H421" s="9" t="n"/>
       <c r="I421" s="9" t="n"/>
       <c r="K421" s="9" t="n"/>
     </row>
     <row r="422">
-      <c r="G422" t="n">
-        <v>10</v>
-      </c>
       <c r="H422" s="9" t="n"/>
       <c r="I422" s="9" t="n"/>
       <c r="K422" s="9" t="n"/>
     </row>
     <row r="423">
-      <c r="G423" t="n">
-        <v>10</v>
-      </c>
       <c r="H423" s="9" t="n"/>
       <c r="I423" s="9" t="n"/>
       <c r="K423" s="9" t="n"/>
     </row>
     <row r="424">
-      <c r="G424" t="n">
-        <v>10</v>
-      </c>
       <c r="H424" s="9" t="n"/>
       <c r="I424" s="9" t="n"/>
       <c r="K424" s="9" t="n"/>
     </row>
     <row r="425">
-      <c r="G425" t="n">
-        <v>10</v>
-      </c>
       <c r="H425" s="9" t="n"/>
       <c r="I425" s="9" t="n"/>
       <c r="K425" s="9" t="n"/>
     </row>
     <row r="426">
-      <c r="G426" t="n">
-        <v>10</v>
-      </c>
       <c r="H426" s="9" t="n"/>
       <c r="I426" s="9" t="n"/>
       <c r="K426" s="9" t="n"/>
     </row>
     <row r="427">
-      <c r="G427" t="n">
-        <v>10</v>
-      </c>
       <c r="H427" s="9" t="n"/>
       <c r="I427" s="9" t="n"/>
       <c r="K427" s="9" t="n"/>
     </row>
     <row r="428">
-      <c r="G428" t="n">
-        <v>10</v>
-      </c>
       <c r="H428" s="9" t="n"/>
       <c r="I428" s="9" t="n"/>
       <c r="K428" s="9" t="n"/>
     </row>
     <row r="429">
-      <c r="G429" t="n">
-        <v>10</v>
-      </c>
       <c r="H429" s="9" t="n"/>
       <c r="I429" s="9" t="n"/>
       <c r="K429" s="9" t="n"/>
     </row>
     <row r="430">
-      <c r="G430" t="n">
-        <v>10</v>
-      </c>
       <c r="H430" s="9" t="n"/>
       <c r="I430" s="9" t="n"/>
       <c r="K430" s="9" t="n"/>
     </row>
     <row r="431">
-      <c r="G431" t="n">
-        <v>10</v>
-      </c>
       <c r="H431" s="9" t="n"/>
       <c r="I431" s="9" t="n"/>
       <c r="K431" s="9" t="n"/>
     </row>
     <row r="432">
-      <c r="G432" t="n">
-        <v>10</v>
-      </c>
       <c r="H432" s="9" t="n"/>
       <c r="I432" s="9" t="n"/>
       <c r="K432" s="9" t="n"/>
     </row>
     <row r="433">
-      <c r="G433" t="n">
-        <v>10</v>
-      </c>
       <c r="H433" s="9" t="n"/>
       <c r="I433" s="9" t="n"/>
       <c r="K433" s="9" t="n"/>
     </row>
     <row r="434">
-      <c r="G434" t="n">
-        <v>10</v>
-      </c>
       <c r="H434" s="9" t="n"/>
       <c r="I434" s="9" t="n"/>
       <c r="K434" s="9" t="n"/>
     </row>
     <row r="435">
-      <c r="G435" t="n">
-        <v>10</v>
-      </c>
       <c r="H435" s="9" t="n"/>
       <c r="I435" s="9" t="n"/>
       <c r="K435" s="9" t="n"/>
     </row>
     <row r="436">
-      <c r="G436" t="n">
-        <v>10</v>
-      </c>
       <c r="H436" s="9" t="n"/>
       <c r="I436" s="9" t="n"/>
       <c r="K436" s="9" t="n"/>
     </row>
     <row r="437">
-      <c r="G437" t="n">
-        <v>10</v>
-      </c>
       <c r="H437" s="9" t="n"/>
       <c r="I437" s="9" t="n"/>
       <c r="K437" s="9" t="n"/>
     </row>
     <row r="438">
-      <c r="G438" t="n">
-        <v>10</v>
-      </c>
       <c r="H438" s="9" t="n"/>
       <c r="I438" s="9" t="n"/>
       <c r="K438" s="9" t="n"/>
     </row>
     <row r="439">
-      <c r="G439" t="n">
-        <v>10</v>
-      </c>
       <c r="H439" s="9" t="n"/>
       <c r="I439" s="9" t="n"/>
       <c r="K439" s="9" t="n"/>
     </row>
     <row r="440">
-      <c r="G440" t="n">
-        <v>10</v>
-      </c>
       <c r="H440" s="9" t="n"/>
       <c r="I440" s="9" t="n"/>
       <c r="K440" s="9" t="n"/>
     </row>
     <row r="441">
-      <c r="G441" t="n">
-        <v>10</v>
-      </c>
       <c r="H441" s="9" t="n"/>
       <c r="I441" s="9" t="n"/>
       <c r="K441" s="9" t="n"/>
     </row>
     <row r="442">
-      <c r="G442" t="n">
-        <v>10</v>
-      </c>
       <c r="H442" s="9" t="n"/>
       <c r="I442" s="9" t="n"/>
       <c r="K442" s="9" t="n"/>
     </row>
     <row r="443">
-      <c r="G443" t="n">
-        <v>10</v>
-      </c>
       <c r="H443" s="9" t="n"/>
       <c r="I443" s="9" t="n"/>
       <c r="K443" s="9" t="n"/>
     </row>
     <row r="444">
-      <c r="G444" t="n">
-        <v>10</v>
-      </c>
       <c r="H444" s="9" t="n"/>
       <c r="I444" s="9" t="n"/>
       <c r="K444" s="9" t="n"/>
     </row>
     <row r="445">
-      <c r="G445" t="n">
-        <v>10</v>
-      </c>
       <c r="H445" s="9" t="n"/>
       <c r="I445" s="9" t="n"/>
       <c r="K445" s="9" t="n"/>
     </row>
     <row r="446">
-      <c r="G446" t="n">
-        <v>10</v>
-      </c>
       <c r="H446" s="9" t="n"/>
       <c r="I446" s="9" t="n"/>
       <c r="K446" s="9" t="n"/>
     </row>
     <row r="447">
-      <c r="G447" t="n">
-        <v>10</v>
-      </c>
       <c r="H447" s="9" t="n"/>
       <c r="I447" s="9" t="n"/>
       <c r="K447" s="9" t="n"/>
     </row>
     <row r="448">
-      <c r="G448" t="n">
-        <v>10</v>
-      </c>
       <c r="H448" s="9" t="n"/>
       <c r="I448" s="9" t="n"/>
       <c r="K448" s="9" t="n"/>
     </row>
     <row r="449">
-      <c r="G449" t="n">
-        <v>10</v>
-      </c>
       <c r="H449" s="9" t="n"/>
       <c r="I449" s="9" t="n"/>
       <c r="K449" s="9" t="n"/>
     </row>
     <row r="450">
-      <c r="G450" t="n">
-        <v>10</v>
-      </c>
       <c r="H450" s="9" t="n"/>
       <c r="I450" s="9" t="n"/>
       <c r="K450" s="9" t="n"/>
     </row>
     <row r="451">
-      <c r="G451" t="n">
-        <v>10</v>
-      </c>
       <c r="H451" s="9" t="n"/>
       <c r="I451" s="9" t="n"/>
       <c r="K451" s="9" t="n"/>
     </row>
     <row r="452">
-      <c r="G452" t="n">
-        <v>10</v>
-      </c>
       <c r="H452" s="9" t="n"/>
       <c r="I452" s="9" t="n"/>
       <c r="K452" s="9" t="n"/>
     </row>
     <row r="453">
-      <c r="G453" t="n">
-        <v>10</v>
-      </c>
       <c r="H453" s="9" t="n"/>
       <c r="I453" s="9" t="n"/>
       <c r="K453" s="9" t="n"/>
     </row>
     <row r="454">
-      <c r="G454" t="n">
-        <v>10</v>
-      </c>
       <c r="H454" s="9" t="n"/>
       <c r="I454" s="9" t="n"/>
       <c r="K454" s="9" t="n"/>
     </row>
     <row r="455">
-      <c r="G455" t="n">
-        <v>10</v>
-      </c>
       <c r="H455" s="9" t="n"/>
       <c r="I455" s="9" t="n"/>
       <c r="K455" s="9" t="n"/>
     </row>
     <row r="456">
-      <c r="G456" t="n">
-        <v>10</v>
-      </c>
       <c r="H456" s="9" t="n"/>
       <c r="I456" s="9" t="n"/>
       <c r="K456" s="9" t="n"/>
     </row>
     <row r="457">
-      <c r="G457" t="n">
-        <v>10</v>
-      </c>
       <c r="H457" s="9" t="n"/>
       <c r="I457" s="9" t="n"/>
       <c r="K457" s="9" t="n"/>
     </row>
     <row r="458">
-      <c r="G458" t="n">
-        <v>10</v>
-      </c>
       <c r="H458" s="9" t="n"/>
       <c r="I458" s="9" t="n"/>
       <c r="K458" s="9" t="n"/>
     </row>
     <row r="459">
-      <c r="G459" t="n">
-        <v>10</v>
-      </c>
       <c r="H459" s="9" t="n"/>
       <c r="I459" s="9" t="n"/>
       <c r="K459" s="9" t="n"/>
     </row>
     <row r="460">
-      <c r="G460" t="n">
-        <v>10</v>
-      </c>
       <c r="H460" s="9" t="n"/>
       <c r="I460" s="9" t="n"/>
       <c r="K460" s="9" t="n"/>
     </row>
     <row r="461">
-      <c r="G461" t="n">
-        <v>10</v>
-      </c>
       <c r="H461" s="9" t="n"/>
       <c r="I461" s="9" t="n"/>
       <c r="K461" s="9" t="n"/>
     </row>
     <row r="462">
-      <c r="G462" t="n">
-        <v>10</v>
-      </c>
       <c r="H462" s="9" t="n"/>
       <c r="I462" s="9" t="n"/>
       <c r="K462" s="9" t="n"/>
     </row>
     <row r="463">
-      <c r="G463" t="n">
-        <v>10</v>
-      </c>
       <c r="H463" s="9" t="n"/>
       <c r="I463" s="9" t="n"/>
       <c r="K463" s="9" t="n"/>
     </row>
     <row r="464">
-      <c r="G464" t="n">
-        <v>10</v>
-      </c>
       <c r="H464" s="9" t="n"/>
       <c r="I464" s="9" t="n"/>
       <c r="K464" s="9" t="n"/>
     </row>
     <row r="465">
-      <c r="G465" t="n">
-        <v>10</v>
-      </c>
       <c r="H465" s="9" t="n"/>
       <c r="I465" s="9" t="n"/>
       <c r="K465" s="9" t="n"/>
     </row>
     <row r="466">
-      <c r="G466" t="n">
-        <v>10</v>
-      </c>
       <c r="H466" s="9" t="n"/>
       <c r="I466" s="9" t="n"/>
       <c r="K466" s="9" t="n"/>
     </row>
     <row r="467">
-      <c r="G467" t="n">
-        <v>10</v>
-      </c>
       <c r="H467" s="9" t="n"/>
       <c r="I467" s="9" t="n"/>
       <c r="K467" s="9" t="n"/>
     </row>
     <row r="468">
-      <c r="G468" t="n">
-        <v>10</v>
-      </c>
       <c r="H468" s="9" t="n"/>
       <c r="I468" s="9" t="n"/>
       <c r="K468" s="9" t="n"/>
     </row>
     <row r="469">
-      <c r="G469" t="n">
-        <v>10</v>
-      </c>
       <c r="H469" s="9" t="n"/>
       <c r="I469" s="9" t="n"/>
       <c r="K469" s="9" t="n"/>
     </row>
     <row r="470">
-      <c r="G470" t="n">
-        <v>10</v>
-      </c>
       <c r="H470" s="9" t="n"/>
       <c r="I470" s="9" t="n"/>
       <c r="K470" s="9" t="n"/>
     </row>
     <row r="471">
-      <c r="G471" t="n">
-        <v>10</v>
-      </c>
       <c r="H471" s="9" t="n"/>
       <c r="I471" s="9" t="n"/>
       <c r="K471" s="9" t="n"/>
     </row>
     <row r="472">
-      <c r="G472" t="n">
-        <v>10</v>
-      </c>
       <c r="H472" s="9" t="n"/>
       <c r="I472" s="9" t="n"/>
       <c r="K472" s="9" t="n"/>
     </row>
     <row r="473">
-      <c r="G473" t="n">
-        <v>10</v>
-      </c>
       <c r="H473" s="9" t="n"/>
       <c r="I473" s="9" t="n"/>
       <c r="K473" s="9" t="n"/>
     </row>
     <row r="474">
-      <c r="G474" t="n">
-        <v>10</v>
-      </c>
       <c r="H474" s="9" t="n"/>
       <c r="I474" s="9" t="n"/>
       <c r="K474" s="9" t="n"/>
     </row>
     <row r="475">
-      <c r="G475" t="n">
-        <v>10</v>
-      </c>
       <c r="H475" s="9" t="n"/>
       <c r="I475" s="9" t="n"/>
       <c r="K475" s="9" t="n"/>
     </row>
     <row r="476">
-      <c r="G476" t="n">
-        <v>10</v>
-      </c>
       <c r="H476" s="9" t="n"/>
       <c r="I476" s="9" t="n"/>
       <c r="K476" s="9" t="n"/>
     </row>
     <row r="477">
-      <c r="G477" t="n">
-        <v>10</v>
-      </c>
       <c r="H477" s="9" t="n"/>
       <c r="I477" s="9" t="n"/>
       <c r="K477" s="9" t="n"/>
     </row>
     <row r="478">
-      <c r="G478" t="n">
-        <v>10</v>
-      </c>
       <c r="H478" s="9" t="n"/>
       <c r="I478" s="9" t="n"/>
       <c r="K478" s="9" t="n"/>
     </row>
     <row r="479">
-      <c r="G479" t="n">
-        <v>10</v>
-      </c>
       <c r="H479" s="9" t="n"/>
       <c r="I479" s="9" t="n"/>
       <c r="K479" s="9" t="n"/>
     </row>
     <row r="480">
-      <c r="G480" t="n">
-        <v>10</v>
-      </c>
       <c r="H480" s="9" t="n"/>
       <c r="I480" s="9" t="n"/>
       <c r="K480" s="9" t="n"/>
     </row>
     <row r="481">
-      <c r="G481" t="n">
-        <v>10</v>
-      </c>
       <c r="H481" s="9" t="n"/>
       <c r="I481" s="9" t="n"/>
       <c r="K481" s="9" t="n"/>
     </row>
     <row r="482">
-      <c r="G482" t="n">
-        <v>10</v>
-      </c>
       <c r="H482" s="9" t="n"/>
       <c r="I482" s="9" t="n"/>
       <c r="K482" s="9" t="n"/>
     </row>
     <row r="483">
-      <c r="G483" t="n">
-        <v>10</v>
-      </c>
       <c r="H483" s="9" t="n"/>
       <c r="I483" s="9" t="n"/>
       <c r="K483" s="9" t="n"/>
     </row>
     <row r="484">
-      <c r="G484" t="n">
-        <v>10</v>
-      </c>
       <c r="H484" s="9" t="n"/>
       <c r="I484" s="9" t="n"/>
       <c r="K484" s="9" t="n"/>
     </row>
     <row r="485">
-      <c r="G485" t="n">
-        <v>10</v>
-      </c>
       <c r="H485" s="9" t="n"/>
       <c r="I485" s="9" t="n"/>
       <c r="K485" s="9" t="n"/>
     </row>
     <row r="486">
-      <c r="G486" t="n">
-        <v>10</v>
-      </c>
       <c r="H486" s="9" t="n"/>
       <c r="I486" s="9" t="n"/>
       <c r="K486" s="9" t="n"/>
     </row>
     <row r="487">
-      <c r="G487" t="n">
-        <v>10</v>
-      </c>
       <c r="H487" s="9" t="n"/>
       <c r="I487" s="9" t="n"/>
       <c r="K487" s="9" t="n"/>
     </row>
     <row r="488">
-      <c r="G488" t="n">
-        <v>10</v>
-      </c>
       <c r="H488" s="9" t="n"/>
       <c r="I488" s="9" t="n"/>
       <c r="K488" s="9" t="n"/>
     </row>
     <row r="489">
-      <c r="G489" t="n">
-        <v>10</v>
-      </c>
       <c r="H489" s="9" t="n"/>
       <c r="I489" s="9" t="n"/>
       <c r="K489" s="9" t="n"/>
     </row>
     <row r="490">
-      <c r="G490" t="n">
-        <v>10</v>
-      </c>
       <c r="H490" s="9" t="n"/>
       <c r="I490" s="9" t="n"/>
       <c r="K490" s="9" t="n"/>
     </row>
     <row r="491">
-      <c r="G491" t="n">
-        <v>10</v>
-      </c>
       <c r="H491" s="9" t="n"/>
       <c r="I491" s="9" t="n"/>
       <c r="K491" s="9" t="n"/>
     </row>
     <row r="492">
-      <c r="G492" t="n">
-        <v>10</v>
-      </c>
       <c r="H492" s="9" t="n"/>
       <c r="I492" s="9" t="n"/>
       <c r="K492" s="9" t="n"/>
     </row>
     <row r="493">
-      <c r="G493" t="n">
-        <v>10</v>
-      </c>
       <c r="H493" s="9" t="n"/>
       <c r="I493" s="9" t="n"/>
       <c r="K493" s="9" t="n"/>
     </row>
     <row r="494">
-      <c r="G494" t="n">
-        <v>10</v>
-      </c>
       <c r="H494" s="9" t="n"/>
       <c r="I494" s="9" t="n"/>
       <c r="K494" s="9" t="n"/>
     </row>
     <row r="495">
-      <c r="G495" t="n">
-        <v>10</v>
-      </c>
       <c r="H495" s="9" t="n"/>
       <c r="I495" s="9" t="n"/>
       <c r="K495" s="9" t="n"/>
     </row>
     <row r="496">
-      <c r="G496" t="n">
-        <v>10</v>
-      </c>
       <c r="H496" s="9" t="n"/>
       <c r="I496" s="9" t="n"/>
       <c r="K496" s="9" t="n"/>
     </row>
     <row r="497">
-      <c r="G497" t="n">
-        <v>10</v>
-      </c>
       <c r="H497" s="9" t="n"/>
       <c r="I497" s="9" t="n"/>
       <c r="K497" s="9" t="n"/>
     </row>
     <row r="498">
-      <c r="G498" t="n">
-        <v>10</v>
-      </c>
       <c r="H498" s="9" t="n"/>
       <c r="I498" s="9" t="n"/>
       <c r="K498" s="9" t="n"/>
     </row>
     <row r="499">
-      <c r="G499" t="n">
-        <v>10</v>
-      </c>
       <c r="H499" s="9" t="n"/>
       <c r="I499" s="9" t="n"/>
       <c r="K499" s="9" t="n"/>
     </row>
     <row r="500">
-      <c r="G500" t="n">
-        <v>10</v>
-      </c>
       <c r="H500" s="9" t="n"/>
       <c r="I500" s="9" t="n"/>
       <c r="K500" s="9" t="n"/>
@@ -5438,9 +3961,7 @@
       <c r="K2" s="7" t="n"/>
       <c r="L2" s="7" t="n"/>
       <c r="M2" s="7" t="n"/>
-      <c r="N2" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="N2" s="6" t="n"/>
       <c r="O2" s="8" t="n"/>
       <c r="P2" s="6" t="n"/>
     </row>
@@ -5506,9 +4027,7 @@
           <t>brought는 '가져왔다'예요.</t>
         </is>
       </c>
-      <c r="N3" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="N3" s="6" t="n"/>
       <c r="O3" s="8" t="n"/>
       <c r="P3" s="6" t="n"/>
     </row>

</xml_diff>